<commit_message>
Latest changes on 12Aug2026
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -1379,7 +1379,7 @@
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://staging.im-aam.com/</v>
+        <v>https://im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1531,7 +1531,7 @@
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://staging.im-aam.com/</v>
+        <v>https://im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1707,7 +1707,7 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Latest changes on 14Aug2026
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -1379,7 +1379,7 @@
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://staging.im-aam.com/</v>
+        <v>https://im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1531,7 +1531,7 @@
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://staging.im-aam.com/</v>
+        <v>https://im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1707,7 +1707,7 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Latest changes on 17Aug2026
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="5"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
-    <sheet name="configMobile" sheetId="1" r:id="rId1"/>
-    <sheet name="permitFlow" sheetId="2" r:id="rId2"/>
-    <sheet name="testFlow" sheetId="3" r:id="rId3"/>
-    <sheet name="Main" sheetId="4" r:id="rId4"/>
+    <sheet name="configMobile" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="permitFlow" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="testFlow" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Main" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="144525" iterateDelta="1E-4"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -24,347 +25,351 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="112">
   <si>
-    <t>Device Name</t>
-  </si>
-  <si>
-    <t>Platform Name</t>
-  </si>
-  <si>
-    <t>Platform Version</t>
-  </si>
-  <si>
-    <t>Automation Name</t>
-  </si>
-  <si>
-    <t>Skip Unlock</t>
-  </si>
-  <si>
-    <t>AVD Launch Timeout</t>
-  </si>
-  <si>
-    <t>Ensure Webview Have Pages</t>
-  </si>
-  <si>
-    <t>Native Web Screenshot</t>
-  </si>
-  <si>
-    <t>New Command Timeout</t>
-  </si>
-  <si>
-    <t>Connect Hardware Keyboard</t>
-  </si>
-  <si>
-    <t>Unicoded Keyboard</t>
-  </si>
-  <si>
-    <t>Reset Keyboard</t>
-  </si>
-  <si>
-    <t>No Reset</t>
-  </si>
-  <si>
-    <t>App Package</t>
-  </si>
-  <si>
-    <t>App Activity</t>
-  </si>
-  <si>
-    <t>Adb Exec Timeout</t>
-  </si>
-  <si>
-    <t>Client Company</t>
-  </si>
-  <si>
-    <t>sdk_gphone64_x86_64</t>
-  </si>
-  <si>
-    <t>Android</t>
-  </si>
-  <si>
-    <t>UiAutomator2</t>
-  </si>
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>false</t>
-  </si>
-  <si>
-    <t>com.app.acompletions</t>
-  </si>
-  <si>
-    <t>com.commissioning.ui.splash.SplashActivity</t>
-  </si>
-  <si>
-    <t>Android SDK built for x86</t>
-  </si>
-  <si>
-    <t>Pixel C</t>
-  </si>
-  <si>
-    <t>Redmi26</t>
-  </si>
-  <si>
-    <t>8.1.0</t>
-  </si>
-  <si>
-    <t>Environment URL</t>
-  </si>
-  <si>
-    <t>Project Name</t>
-  </si>
-  <si>
-    <t>L2 User Credentials</t>
-  </si>
-  <si>
-    <t>Permit Holder Credentials</t>
-  </si>
-  <si>
-    <t>L4 User Credentials</t>
-  </si>
-  <si>
-    <t>PCO User Credentials</t>
-  </si>
-  <si>
-    <t>Permit Approver (L4) Name</t>
-  </si>
-  <si>
-    <t>Projectr Admin Credentials</t>
-  </si>
-  <si>
-    <t>Discipline</t>
-  </si>
-  <si>
-    <t>http://cybuild.devpress.net</t>
-  </si>
-  <si>
-    <t>Brave</t>
-  </si>
-  <si>
-    <t>todd.beck@example.com/123456</t>
-  </si>
-  <si>
-    <t>julie.cole@example.com/123456</t>
-  </si>
-  <si>
-    <t>noah.poulsen@example.com/123456</t>
-  </si>
-  <si>
-    <t>Julie Cole</t>
-  </si>
-  <si>
-    <t>dhaval.barot@indianic.com/123456</t>
-  </si>
-  <si>
-    <t>tom@mac-24.com/Test@123</t>
-  </si>
-  <si>
-    <t>john@mac-24.com/123456</t>
-  </si>
-  <si>
-    <t>kevin@mac-24.com/123456</t>
-  </si>
-  <si>
-    <t>Niall Stenson</t>
-  </si>
-  <si>
-    <t>QA Manager Credentials</t>
-  </si>
-  <si>
-    <t>Project Admin Credentials</t>
-  </si>
-  <si>
-    <t>Supervisor Credentials</t>
-  </si>
-  <si>
-    <t>Engineer Credentials</t>
-  </si>
-  <si>
-    <t>Technical Admin Credentials</t>
-  </si>
-  <si>
-    <t>Super Admin Credentials</t>
-  </si>
-  <si>
-    <t>https://im-aam.com/</t>
-  </si>
-  <si>
-    <t>UGL</t>
-  </si>
-  <si>
-    <t>Hunter Power Project</t>
-  </si>
-  <si>
-    <t>anand.sharma+021501@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>anna.miller@example.com/123456</t>
-  </si>
-  <si>
-    <t>qaapprover1.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>qaapprover2.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>jaydeep.d+040420239@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>Ad Sd</t>
-  </si>
-  <si>
-    <t>coUser1.15july2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>supervisor.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>engineer.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>technicaladmin.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>admin@cybuild.com.au/Commsite12#</t>
-  </si>
-  <si>
-    <t>E&amp;IC</t>
-  </si>
-  <si>
-    <t>https://staging.im-aam.com/</t>
-  </si>
-  <si>
-    <t>hiren.joshi+L201PH@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>matt@acompletions.com/123456</t>
-  </si>
-  <si>
-    <t>https://dev.cybuild.com.au/</t>
-  </si>
-  <si>
-    <t>https://cybuild.com.au</t>
-  </si>
-  <si>
-    <t>Demo Project</t>
-  </si>
-  <si>
-    <t>hiren.joshi+L401PA@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>hiren.joshi+L701PCO@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>HirenEdited Joshi L4 01 PAEdited</t>
-  </si>
-  <si>
-    <t>anand.sharma+20230501@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>987671231/Test@123</t>
-  </si>
-  <si>
-    <t>987789654/Test@123</t>
-  </si>
-  <si>
-    <t>789123321/Test@123</t>
-  </si>
-  <si>
-    <t>15feb-1@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>test02152023120271@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>test021520231202899@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>L4 User</t>
-  </si>
-  <si>
-    <t>qaapprover3@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>qaapprover4@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>qaapprover1@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>qaapprover2@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>https://cybuild.devpress.net</t>
-  </si>
-  <si>
-    <t>permitwriter@example.com/Test@123</t>
-  </si>
-  <si>
-    <t>1May2023-l2@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>1May2023-l4@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>1May2023-pco@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>1May2023 L4</t>
-  </si>
-  <si>
-    <t>acompletions@admin.com/123456</t>
-  </si>
-  <si>
-    <t>sara.johansen@example.com/123456</t>
-  </si>
-  <si>
-    <t>https://dev-ugl.cybuild.com.au/</t>
-  </si>
-  <si>
-    <t>Work Pack Demo</t>
-  </si>
-  <si>
-    <t>https://dev-app.cybuild.com.au/</t>
-  </si>
-  <si>
-    <t>John Holland</t>
-  </si>
-  <si>
-    <t>WestConnex 3B</t>
-  </si>
-  <si>
-    <t>anand.sharma+040420232@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>https://app.cybuild.com.au</t>
-  </si>
-  <si>
-    <t>permit.writer@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>permit.approver@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>permit.pco@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>Permit Approver</t>
-  </si>
-  <si>
-    <t>anand.sharma+2023022401@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>matt@cybuild.com.au/Commsite12#</t>
-  </si>
-  <si>
-    <t>quoisoforafei-1118@yopmail.com/Test@123</t>
+    <t xml:space="preserve">Device Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Platform Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Platform Version</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automation Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skip Unlock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVD Launch Timeout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ensure Webview Have Pages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Native Web Screenshot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New Command Timeout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Connect Hardware Keyboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unicoded Keyboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reset Keyboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Reset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App Package</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App Activity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adb Exec Timeout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Client Company</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdk_gphone64_x86_64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Android</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UiAutomator2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">true</t>
+  </si>
+  <si>
+    <t xml:space="preserve">false</t>
+  </si>
+  <si>
+    <t xml:space="preserve">com.app.acompletions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">com.commissioning.ui.splash.SplashActivity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Android SDK built for x86</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pixel C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redmi26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.1.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Environment URL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L2 User Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit Holder Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L4 User Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCO User Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit Approver (L4) Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projectr Admin Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discipline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://cybuild.devpress.net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brave</t>
+  </si>
+  <si>
+    <t xml:space="preserve">todd.beck@example.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">julie.cole@example.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">noah.poulsen@example.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Julie Cole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dhaval.barot@indianic.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tom@mac-24.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">john@mac-24.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kevin@mac-24.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niall Stenson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QA Manager Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project Admin Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supervisor Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engineer Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technical Admin Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Admin Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://im-aam.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UGL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hunter Power Project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">anand.sharma+021501@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">anna.miller@example.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qaapprover1.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qaapprover2.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jaydeep.d+040420239@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ad Sd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">coUser1.15july2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supervisor.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">engineer.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">technicaladmin.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">admin@cybuild.com.au/Commsite12#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E&amp;IC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://staging.im-aam.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hiren.joshi+L201PH@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">matt@acompletions.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://dev.cybuild.com.au/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://cybuild.com.au</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demo Project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hiren.joshi+L401PA@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hiren.joshi+L701PCO@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HirenEdited Joshi L4 01 PAEdited</t>
+  </si>
+  <si>
+    <t xml:space="preserve">anand.sharma+20230501@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">987671231/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">987789654/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">789123321/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15feb-1@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test02152023120271@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test021520231202899@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L4 User</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qaapprover3@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qaapprover4@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qaapprover1@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qaapprover2@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://cybuild.devpress.net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">permitwriter@example.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1May2023-l2@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1May2023-l4@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1May2023-pco@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1May2023 L4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">acompletions@admin.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sara.johansen@example.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://dev-ugl.cybuild.com.au/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Work Pack Demo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://dev-app.cybuild.com.au/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">John Holland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WestConnex 3B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">anand.sharma+040420232@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://app.cybuild.com.au</t>
+  </si>
+  <si>
+    <t xml:space="preserve">permit.writer@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">permit.approver@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">permit.pco@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit Approver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">anand.sharma+2023022401@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">matt@cybuild.com.au/Commsite12#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quoisoforafei-1118@yopmail.com/Test@123</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="@"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -373,7 +378,22 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -381,7 +401,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <u/>
+      <u val="single"/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
@@ -398,47 +418,84 @@
     </fill>
   </fills>
   <borders count="2">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+  <cellStyleXfs count="21">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -497,26 +554,13 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -558,12 +602,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Calibri Light" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -595,7 +639,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -619,7 +663,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -679,41 +723,42 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:Q35"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="23.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="27" style="1" customWidth="1"/>
-    <col min="8" max="8" width="22.28515625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="22.85546875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26.7109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="18.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15" style="1" customWidth="1"/>
-    <col min="13" max="13" width="9" style="1" customWidth="1"/>
-    <col min="14" max="14" width="21.5703125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="41" style="1" customWidth="1"/>
-    <col min="16" max="16" width="17" style="1" customWidth="1"/>
-    <col min="17" max="17" width="15.140625" style="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="22.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="26.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="18.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="21.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="15.14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -766,14 +811,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="1" t="n">
         <v>14</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -782,7 +827,7 @@
       <c r="E2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G2" s="4" t="s">
@@ -791,7 +836,7 @@
       <c r="H2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J2" s="4" t="s">
@@ -812,27 +857,27 @@
       <c r="O2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="1" t="n">
         <v>60000</v>
       </c>
       <c r="Q2" s="1" t="str">
-        <f>Main!B2</f>
+        <f aca="false">Main!B2</f>
         <v>UGL</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C3" s="1">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C3" s="1" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="1" t="n">
         <v>13</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -841,7 +886,7 @@
       <c r="E4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G4" s="4" t="s">
@@ -850,7 +895,7 @@
       <c r="H4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J4" s="4" t="s">
@@ -872,19 +917,19 @@
         <v>23</v>
       </c>
       <c r="P4" s="4"/>
-      <c r="Q4" s="1">
-        <f>Main!B4</f>
+      <c r="Q4" s="1" t="n">
+        <f aca="false">Main!B4</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="1" t="n">
         <v>11</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -893,7 +938,7 @@
       <c r="E6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G6" s="4" t="s">
@@ -902,7 +947,7 @@
       <c r="H6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J6" s="4" t="s">
@@ -925,14 +970,14 @@
       </c>
       <c r="P6" s="4"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="1" t="n">
         <v>13</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -941,7 +986,7 @@
       <c r="E10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G10" s="4" t="s">
@@ -950,7 +995,7 @@
       <c r="H10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J10" s="4" t="s">
@@ -973,14 +1018,14 @@
       </c>
       <c r="P10" s="4"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="1" t="n">
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -989,7 +1034,7 @@
       <c r="E14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F14" s="1">
+      <c r="F14" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G14" s="4" t="s">
@@ -998,7 +1043,7 @@
       <c r="H14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J14" s="4" t="s">
@@ -1021,14 +1066,14 @@
       </c>
       <c r="P14" s="4"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="1" t="n">
         <v>13</v>
       </c>
       <c r="D20" s="1" t="s">
@@ -1037,7 +1082,7 @@
       <c r="E20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F20" s="1">
+      <c r="F20" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G20" s="4" t="s">
@@ -1046,7 +1091,7 @@
       <c r="H20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I20" s="1">
+      <c r="I20" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J20" s="4" t="s">
@@ -1069,14 +1114,14 @@
       </c>
       <c r="P20" s="4"/>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C23" s="1">
+      <c r="C23" s="1" t="n">
         <v>13</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -1085,7 +1130,7 @@
       <c r="E23" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F23" s="1">
+      <c r="F23" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G23" s="4" t="s">
@@ -1094,7 +1139,7 @@
       <c r="H23" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I23" s="1">
+      <c r="I23" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J23" s="4" t="s">
@@ -1116,19 +1161,19 @@
         <v>23</v>
       </c>
       <c r="P23" s="4"/>
-      <c r="Q23" s="1">
-        <f>Main!B23</f>
+      <c r="Q23" s="1" t="n">
+        <f aca="false">Main!B23</f>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25" s="1" t="n">
         <v>12</v>
       </c>
       <c r="D25" s="1" t="s">
@@ -1137,7 +1182,7 @@
       <c r="E25" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F25" s="1">
+      <c r="F25" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G25" s="4" t="s">
@@ -1146,7 +1191,7 @@
       <c r="H25" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I25" s="1">
+      <c r="I25" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J25" s="4" t="s">
@@ -1169,7 +1214,7 @@
       </c>
       <c r="P25" s="4"/>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -1185,7 +1230,7 @@
       <c r="E28" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F28" s="1">
+      <c r="F28" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G28" s="4" t="s">
@@ -1194,7 +1239,7 @@
       <c r="H28" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I28" s="1">
+      <c r="I28" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J28" s="4" t="s">
@@ -1216,19 +1261,19 @@
         <v>23</v>
       </c>
       <c r="P28" s="4"/>
-      <c r="Q28" s="1">
-        <f>Main!B28</f>
+      <c r="Q28" s="1" t="n">
+        <f aca="false">Main!B28</f>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="1">
+      <c r="C33" s="1" t="n">
         <v>8</v>
       </c>
       <c r="D33" s="1" t="s">
@@ -1237,7 +1282,7 @@
       <c r="E33" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F33" s="1">
+      <c r="F33" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G33" s="4" t="s">
@@ -1246,7 +1291,7 @@
       <c r="H33" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I33" s="1">
+      <c r="I33" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J33" s="4" t="s">
@@ -1268,19 +1313,19 @@
         <v>23</v>
       </c>
       <c r="P33" s="4"/>
-      <c r="Q33" s="1">
-        <f>Main!B33</f>
+      <c r="Q33" s="1" t="n">
+        <f aca="false">Main!B33</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C35" s="1">
+      <c r="C35" s="1" t="n">
         <v>12</v>
       </c>
       <c r="D35" s="1" t="s">
@@ -1289,7 +1334,7 @@
       <c r="E35" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F35" s="1">
+      <c r="F35" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G35" s="4" t="s">
@@ -1298,7 +1343,7 @@
       <c r="H35" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I35" s="1">
+      <c r="I35" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J35" s="4" t="s">
@@ -1321,33 +1366,41 @@
       </c>
       <c r="P35" s="4"/>
       <c r="Q35" s="1" t="str">
-        <f>Main!B35</f>
+        <f aca="false">Main!B35</f>
         <v>UGL</v>
       </c>
     </row>
   </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="26.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="34.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="31.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="30.7109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="34.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="30.42578125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="46.28515625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" style="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="31.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="30.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="34.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="30.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="46.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.71"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -1376,45 +1429,45 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="str">
-        <f>Main!A2</f>
+        <f aca="false">Main!A2</f>
         <v>https://im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
-        <f>Main!B2</f>
+        <f aca="false">Main!B2</f>
         <v>UGL</v>
       </c>
       <c r="C2" s="1" t="str">
-        <f>Main!D2</f>
+        <f aca="false">Main!D2</f>
         <v>anand.sharma+021501@indianic.com/Test@123</v>
       </c>
       <c r="D2" s="1" t="str">
-        <f>Main!E2</f>
+        <f aca="false">Main!E2</f>
         <v>anna.miller@example.com/123456</v>
       </c>
       <c r="E2" s="1" t="str">
-        <f>Main!F2</f>
+        <f aca="false">Main!F2</f>
         <v>qaapprover1.27may2025@yopmail.com/Test@123</v>
       </c>
       <c r="F2" s="1" t="str">
-        <f>Main!H2</f>
+        <f aca="false">Main!H2</f>
         <v>jaydeep.d+040420239@indianic.com/Test@123</v>
       </c>
       <c r="G2" s="1" t="str">
-        <f>Main!I2</f>
+        <f aca="false">Main!I2</f>
         <v>Ad Sd</v>
       </c>
       <c r="H2" s="1" t="str">
-        <f>Main!J2</f>
+        <f aca="false">Main!J2</f>
         <v>coUser1.15july2025@yopmail.com/Test@123</v>
       </c>
       <c r="I2" s="1" t="str">
-        <f>Main!O2</f>
+        <f aca="false">Main!O2</f>
         <v>E&amp;IC</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>37</v>
       </c>
@@ -1437,7 +1490,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C13" s="1" t="s">
         <v>44</v>
       </c>
@@ -1453,35 +1506,43 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A11" r:id="rId1"/>
+    <hyperlink ref="A11" r:id="rId1" display="http://cybuild.devpress.net"/>
   </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:O13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16" style="1" customWidth="1"/>
-    <col min="4" max="4" width="44.140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="32.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="47.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="48.28515625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="43.5703125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="25.7109375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="40.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="42.85546875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="41.28515625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="46.7109375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="35.5703125" style="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="44.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="32.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="47.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="48.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="43.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="25.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="40.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="42.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="41.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="46.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="35.57"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -1528,69 +1589,69 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="str">
-        <f>Main!A2</f>
+        <f aca="false">Main!A2</f>
         <v>https://im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
-        <f>Main!B2</f>
+        <f aca="false">Main!B2</f>
         <v>UGL</v>
       </c>
       <c r="C2" s="1" t="str">
-        <f>Main!C2</f>
+        <f aca="false">Main!C2</f>
         <v>Hunter Power Project</v>
       </c>
       <c r="D2" s="1" t="str">
-        <f>Main!D2</f>
+        <f aca="false">Main!D2</f>
         <v>anand.sharma+021501@indianic.com/Test@123</v>
       </c>
       <c r="E2" s="1" t="str">
-        <f>Main!E2</f>
+        <f aca="false">Main!E2</f>
         <v>anna.miller@example.com/123456</v>
       </c>
       <c r="F2" s="1" t="str">
-        <f>Main!F2</f>
+        <f aca="false">Main!F2</f>
         <v>qaapprover1.27may2025@yopmail.com/Test@123</v>
       </c>
       <c r="G2" s="1" t="str">
-        <f>Main!G2</f>
+        <f aca="false">Main!G2</f>
         <v>qaapprover2.27may2025@yopmail.com/Test@123</v>
       </c>
       <c r="H2" s="1" t="str">
-        <f>Main!H2</f>
+        <f aca="false">Main!H2</f>
         <v>jaydeep.d+040420239@indianic.com/Test@123</v>
       </c>
       <c r="I2" s="1" t="str">
-        <f>Main!I2</f>
+        <f aca="false">Main!I2</f>
         <v>Ad Sd</v>
       </c>
       <c r="J2" s="1" t="str">
-        <f>Main!J2</f>
+        <f aca="false">Main!J2</f>
         <v>coUser1.15july2025@yopmail.com/Test@123</v>
       </c>
       <c r="K2" s="1" t="str">
-        <f>Main!K2</f>
+        <f aca="false">Main!K2</f>
         <v>supervisor.27may2025@yopmail.com/Test@123</v>
       </c>
       <c r="L2" s="1" t="str">
-        <f>Main!L2</f>
+        <f aca="false">Main!L2</f>
         <v>engineer.27may2025@yopmail.com/Test@123</v>
       </c>
       <c r="M2" s="1" t="str">
-        <f>Main!M2</f>
+        <f aca="false">Main!M2</f>
         <v>technicaladmin.27may2025@yopmail.com/Test@123</v>
       </c>
       <c r="N2" s="1" t="str">
-        <f>Main!N2</f>
+        <f aca="false">Main!N2</f>
         <v>admin@cybuild.com.au/Commsite12#</v>
       </c>
       <c r="O2" s="1" t="str">
-        <f>Main!O2</f>
+        <f aca="false">Main!O2</f>
         <v>E&amp;IC</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>37</v>
       </c>
@@ -1614,7 +1675,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D13" s="1" t="s">
         <v>44</v>
       </c>
@@ -1630,35 +1691,43 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A11" r:id="rId1"/>
+    <hyperlink ref="A11" r:id="rId1" display="http://cybuild.devpress.net"/>
   </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:O49"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="30.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="20.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="48.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="41.42578125" style="1" customWidth="1"/>
-    <col min="6" max="7" width="47.28515625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="43.28515625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="30.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="48.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="43" style="1" customWidth="1"/>
-    <col min="12" max="12" width="41.7109375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="47.28515625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="35.5703125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="10.5703125" style="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="48.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="47.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="43.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="48.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="41.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="47.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="35.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="10.57"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -1705,7 +1774,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>54</v>
       </c>
@@ -1752,7 +1821,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>69</v>
       </c>
@@ -1763,12 +1832,12 @@
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>72</v>
       </c>
@@ -1791,7 +1860,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
         <v>73</v>
       </c>
@@ -1814,7 +1883,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>73</v>
       </c>
@@ -1837,7 +1906,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>73</v>
       </c>
@@ -1860,7 +1929,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D17" s="1" t="s">
         <v>39</v>
       </c>
@@ -1871,7 +1940,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F18" s="1" t="s">
         <v>88</v>
       </c>
@@ -1882,13 +1951,13 @@
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B19" s="5"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
         <v>73</v>
       </c>
@@ -1911,7 +1980,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
         <v>73</v>
       </c>
@@ -1937,7 +2006,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
         <v>72</v>
       </c>
@@ -1969,22 +2038,22 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C32" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
         <v>100</v>
       </c>
@@ -2016,7 +2085,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="1" t="s">
         <v>55</v>
       </c>
@@ -2024,7 +2093,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
         <v>104</v>
       </c>
@@ -2056,12 +2125,12 @@
         <v>67</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C41" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
         <v>100</v>
       </c>
@@ -2096,7 +2165,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
         <v>100</v>
       </c>
@@ -2131,7 +2200,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
         <v>98</v>
       </c>
@@ -2178,45 +2247,50 @@
         <v>68</v>
       </c>
     </row>
-    <row r="49" spans="10:10" x14ac:dyDescent="0.25">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="J49" s="1" t="s">
         <v>110</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1"/>
-    <hyperlink ref="K2" r:id="rId2"/>
-    <hyperlink ref="L2" r:id="rId3"/>
-    <hyperlink ref="M2" r:id="rId4"/>
-    <hyperlink ref="J4" r:id="rId5"/>
-    <hyperlink ref="J6" r:id="rId6"/>
-    <hyperlink ref="F12" r:id="rId7"/>
-    <hyperlink ref="F14" r:id="rId8"/>
-    <hyperlink ref="H14" r:id="rId9"/>
-    <hyperlink ref="J14" r:id="rId10"/>
-    <hyperlink ref="J18" r:id="rId11"/>
-    <hyperlink ref="D24" r:id="rId12"/>
-    <hyperlink ref="F24" r:id="rId13"/>
-    <hyperlink ref="H24" r:id="rId14"/>
-    <hyperlink ref="J24" r:id="rId15"/>
-    <hyperlink ref="A26" r:id="rId16"/>
-    <hyperlink ref="E26" r:id="rId17"/>
-    <hyperlink ref="J26" r:id="rId18"/>
-    <hyperlink ref="A28" r:id="rId19"/>
-    <hyperlink ref="E34" r:id="rId20"/>
-    <hyperlink ref="J34" r:id="rId21"/>
-    <hyperlink ref="E37" r:id="rId22"/>
-    <hyperlink ref="J37" r:id="rId23"/>
-    <hyperlink ref="E43" r:id="rId24"/>
-    <hyperlink ref="J43" r:id="rId25"/>
-    <hyperlink ref="E46" r:id="rId26"/>
-    <hyperlink ref="E48" r:id="rId27"/>
-    <hyperlink ref="K48" r:id="rId28"/>
-    <hyperlink ref="L48" r:id="rId29"/>
-    <hyperlink ref="M48" r:id="rId30"/>
+    <hyperlink ref="E2" r:id="rId1" display="anna.miller@example.com/123456"/>
+    <hyperlink ref="K2" r:id="rId2" display="supervisor.27may2025@yopmail.com/Test@123"/>
+    <hyperlink ref="L2" r:id="rId3" display="engineer.27may2025@yopmail.com/Test@123"/>
+    <hyperlink ref="M2" r:id="rId4" display="technicaladmin.27may2025@yopmail.com/Test@123"/>
+    <hyperlink ref="J4" r:id="rId5" display="matt@acompletions.com/123456"/>
+    <hyperlink ref="J6" r:id="rId6" display="dhaval.barot@indianic.com/123456"/>
+    <hyperlink ref="F12" r:id="rId7" display="987789654/Test@123"/>
+    <hyperlink ref="F14" r:id="rId8" display="test02152023120271@yopmail.com/Test@123"/>
+    <hyperlink ref="H14" r:id="rId9" display="test021520231202899@yopmail.com/Test@123"/>
+    <hyperlink ref="J14" r:id="rId10" display="matt@acompletions.com/123456"/>
+    <hyperlink ref="J18" r:id="rId11" display="dhaval.barot@indianic.com/123456"/>
+    <hyperlink ref="D24" r:id="rId12" display="1May2023-l2@yopmail.com/Test@123"/>
+    <hyperlink ref="F24" r:id="rId13" display="1May2023-l4@yopmail.com/Test@123"/>
+    <hyperlink ref="H24" r:id="rId14" display="1May2023-pco@yopmail.com/Test@123"/>
+    <hyperlink ref="J24" r:id="rId15" display="matt@acompletions.com/123456"/>
+    <hyperlink ref="A26" r:id="rId16" display="https://dev.cybuild.com.au/"/>
+    <hyperlink ref="E26" r:id="rId17" display="anna.miller@example.com/123456"/>
+    <hyperlink ref="J26" r:id="rId18" display="matt@acompletions.com/123456"/>
+    <hyperlink ref="A28" r:id="rId19" display="https://dev.cybuild.com.au/"/>
+    <hyperlink ref="E34" r:id="rId20" display="anna.miller@example.com/123456"/>
+    <hyperlink ref="J34" r:id="rId21" display="matt@acompletions.com/123456"/>
+    <hyperlink ref="E37" r:id="rId22" display="anna.miller@example.com/123456"/>
+    <hyperlink ref="J37" r:id="rId23" display="matt@acompletions.com/123456"/>
+    <hyperlink ref="E43" r:id="rId24" display="anna.miller@example.com/123456"/>
+    <hyperlink ref="J43" r:id="rId25" display="matt@acompletions.com/123456"/>
+    <hyperlink ref="E46" r:id="rId26" display="anna.miller@example.com/123456"/>
+    <hyperlink ref="E48" r:id="rId27" display="anna.miller@example.com/123456"/>
+    <hyperlink ref="K48" r:id="rId28" display="supervisor.27may2025@yopmail.com/Test@123"/>
+    <hyperlink ref="L48" r:id="rId29" display="engineer.27may2025@yopmail.com/Test@123"/>
+    <hyperlink ref="M48" r:id="rId30" display="technicaladmin.27may2025@yopmail.com/Test@123"/>
   </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Latest cahnges on 19 August 2026
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -1,19 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="5"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="3"/>
   </bookViews>
   <sheets>
-    <sheet name="configMobile" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="permitFlow" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="testFlow" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Main" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="configMobile" sheetId="1" r:id="rId1"/>
+    <sheet name="permitFlow" sheetId="2" r:id="rId2"/>
+    <sheet name="testFlow" sheetId="3" r:id="rId3"/>
+    <sheet name="Main" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="144525" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,351 +24,347 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="112">
   <si>
-    <t xml:space="preserve">Device Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Platform Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Platform Version</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Automation Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skip Unlock</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVD Launch Timeout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ensure Webview Have Pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Native Web Screenshot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New Command Timeout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Connect Hardware Keyboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unicoded Keyboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reset Keyboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No Reset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App Package</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App Activity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adb Exec Timeout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Client Company</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sdk_gphone64_x86_64</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Android</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UiAutomator2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">true</t>
-  </si>
-  <si>
-    <t xml:space="preserve">false</t>
-  </si>
-  <si>
-    <t xml:space="preserve">com.app.acompletions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">com.commissioning.ui.splash.SplashActivity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Android SDK built for x86</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pixel C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redmi26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.1.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Environment URL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L2 User Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permit Holder Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L4 User Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PCO User Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permit Approver (L4) Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Projectr Admin Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Discipline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://cybuild.devpress.net</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brave</t>
-  </si>
-  <si>
-    <t xml:space="preserve">todd.beck@example.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">julie.cole@example.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">noah.poulsen@example.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Julie Cole</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dhaval.barot@indianic.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tom@mac-24.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">john@mac-24.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kevin@mac-24.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Niall Stenson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QA Manager Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project Admin Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supervisor Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Engineer Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Technical Admin Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Admin Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://im-aam.com/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UGL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hunter Power Project</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anand.sharma+021501@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anna.miller@example.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">qaapprover1.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">qaapprover2.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jaydeep.d+040420239@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ad Sd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">coUser1.15july2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">supervisor.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">engineer.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">technicaladmin.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">admin@cybuild.com.au/Commsite12#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E&amp;IC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://staging.im-aam.com/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hiren.joshi+L201PH@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">matt@acompletions.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://dev.cybuild.com.au/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://cybuild.com.au</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demo Project</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hiren.joshi+L401PA@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hiren.joshi+L701PCO@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HirenEdited Joshi L4 01 PAEdited</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anand.sharma+20230501@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">987671231/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">987789654/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">789123321/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15feb-1@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test02152023120271@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test021520231202899@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L4 User</t>
-  </si>
-  <si>
-    <t xml:space="preserve">qaapprover3@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">qaapprover4@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">qaapprover1@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">qaapprover2@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://cybuild.devpress.net</t>
-  </si>
-  <si>
-    <t xml:space="preserve">permitwriter@example.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1May2023-l2@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1May2023-l4@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1May2023-pco@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1May2023 L4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">acompletions@admin.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sara.johansen@example.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://dev-ugl.cybuild.com.au/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Work Pack Demo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://dev-app.cybuild.com.au/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">John Holland</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WestConnex 3B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anand.sharma+040420232@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://app.cybuild.com.au</t>
-  </si>
-  <si>
-    <t xml:space="preserve">permit.writer@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">permit.approver@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">permit.pco@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permit Approver</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anand.sharma+2023022401@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">matt@cybuild.com.au/Commsite12#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">quoisoforafei-1118@yopmail.com/Test@123</t>
+    <t>Device Name</t>
+  </si>
+  <si>
+    <t>Platform Name</t>
+  </si>
+  <si>
+    <t>Platform Version</t>
+  </si>
+  <si>
+    <t>Automation Name</t>
+  </si>
+  <si>
+    <t>Skip Unlock</t>
+  </si>
+  <si>
+    <t>AVD Launch Timeout</t>
+  </si>
+  <si>
+    <t>Ensure Webview Have Pages</t>
+  </si>
+  <si>
+    <t>Native Web Screenshot</t>
+  </si>
+  <si>
+    <t>New Command Timeout</t>
+  </si>
+  <si>
+    <t>Connect Hardware Keyboard</t>
+  </si>
+  <si>
+    <t>Unicoded Keyboard</t>
+  </si>
+  <si>
+    <t>Reset Keyboard</t>
+  </si>
+  <si>
+    <t>No Reset</t>
+  </si>
+  <si>
+    <t>App Package</t>
+  </si>
+  <si>
+    <t>App Activity</t>
+  </si>
+  <si>
+    <t>Adb Exec Timeout</t>
+  </si>
+  <si>
+    <t>Client Company</t>
+  </si>
+  <si>
+    <t>sdk_gphone64_x86_64</t>
+  </si>
+  <si>
+    <t>Android</t>
+  </si>
+  <si>
+    <t>UiAutomator2</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t>com.app.acompletions</t>
+  </si>
+  <si>
+    <t>com.commissioning.ui.splash.SplashActivity</t>
+  </si>
+  <si>
+    <t>Android SDK built for x86</t>
+  </si>
+  <si>
+    <t>Pixel C</t>
+  </si>
+  <si>
+    <t>Redmi26</t>
+  </si>
+  <si>
+    <t>8.1.0</t>
+  </si>
+  <si>
+    <t>Environment URL</t>
+  </si>
+  <si>
+    <t>Project Name</t>
+  </si>
+  <si>
+    <t>L2 User Credentials</t>
+  </si>
+  <si>
+    <t>Permit Holder Credentials</t>
+  </si>
+  <si>
+    <t>L4 User Credentials</t>
+  </si>
+  <si>
+    <t>PCO User Credentials</t>
+  </si>
+  <si>
+    <t>Permit Approver (L4) Name</t>
+  </si>
+  <si>
+    <t>Projectr Admin Credentials</t>
+  </si>
+  <si>
+    <t>Discipline</t>
+  </si>
+  <si>
+    <t>http://cybuild.devpress.net</t>
+  </si>
+  <si>
+    <t>Brave</t>
+  </si>
+  <si>
+    <t>todd.beck@example.com/123456</t>
+  </si>
+  <si>
+    <t>julie.cole@example.com/123456</t>
+  </si>
+  <si>
+    <t>noah.poulsen@example.com/123456</t>
+  </si>
+  <si>
+    <t>Julie Cole</t>
+  </si>
+  <si>
+    <t>dhaval.barot@indianic.com/123456</t>
+  </si>
+  <si>
+    <t>tom@mac-24.com/Test@123</t>
+  </si>
+  <si>
+    <t>john@mac-24.com/123456</t>
+  </si>
+  <si>
+    <t>kevin@mac-24.com/123456</t>
+  </si>
+  <si>
+    <t>Niall Stenson</t>
+  </si>
+  <si>
+    <t>QA Manager Credentials</t>
+  </si>
+  <si>
+    <t>Project Admin Credentials</t>
+  </si>
+  <si>
+    <t>Supervisor Credentials</t>
+  </si>
+  <si>
+    <t>Engineer Credentials</t>
+  </si>
+  <si>
+    <t>Technical Admin Credentials</t>
+  </si>
+  <si>
+    <t>Super Admin Credentials</t>
+  </si>
+  <si>
+    <t>https://im-aam.com/</t>
+  </si>
+  <si>
+    <t>UGL</t>
+  </si>
+  <si>
+    <t>Hunter Power Project</t>
+  </si>
+  <si>
+    <t>anand.sharma+021501@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t>anna.miller@example.com/123456</t>
+  </si>
+  <si>
+    <t>qaapprover1.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>qaapprover2.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>jaydeep.d+040420239@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t>Ad Sd</t>
+  </si>
+  <si>
+    <t>coUser1.15july2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>supervisor.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>engineer.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>technicaladmin.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>admin@cybuild.com.au/Commsite12#</t>
+  </si>
+  <si>
+    <t>E&amp;IC</t>
+  </si>
+  <si>
+    <t>https://staging.im-aam.com/</t>
+  </si>
+  <si>
+    <t>hiren.joshi+L201PH@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t>matt@acompletions.com/123456</t>
+  </si>
+  <si>
+    <t>https://dev.cybuild.com.au/</t>
+  </si>
+  <si>
+    <t>https://cybuild.com.au</t>
+  </si>
+  <si>
+    <t>Demo Project</t>
+  </si>
+  <si>
+    <t>hiren.joshi+L401PA@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t>hiren.joshi+L701PCO@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t>HirenEdited Joshi L4 01 PAEdited</t>
+  </si>
+  <si>
+    <t>anand.sharma+20230501@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t>987671231/Test@123</t>
+  </si>
+  <si>
+    <t>987789654/Test@123</t>
+  </si>
+  <si>
+    <t>789123321/Test@123</t>
+  </si>
+  <si>
+    <t>15feb-1@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>test02152023120271@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>test021520231202899@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>L4 User</t>
+  </si>
+  <si>
+    <t>qaapprover3@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>qaapprover4@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>qaapprover1@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>qaapprover2@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>https://cybuild.devpress.net</t>
+  </si>
+  <si>
+    <t>permitwriter@example.com/Test@123</t>
+  </si>
+  <si>
+    <t>1May2023-l2@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>1May2023-l4@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>1May2023-pco@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>1May2023 L4</t>
+  </si>
+  <si>
+    <t>acompletions@admin.com/123456</t>
+  </si>
+  <si>
+    <t>sara.johansen@example.com/123456</t>
+  </si>
+  <si>
+    <t>https://dev-ugl.cybuild.com.au/</t>
+  </si>
+  <si>
+    <t>Work Pack Demo</t>
+  </si>
+  <si>
+    <t>https://dev-app.cybuild.com.au/</t>
+  </si>
+  <si>
+    <t>John Holland</t>
+  </si>
+  <si>
+    <t>WestConnex 3B</t>
+  </si>
+  <si>
+    <t>anand.sharma+040420232@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t>https://app.cybuild.com.au</t>
+  </si>
+  <si>
+    <t>permit.writer@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>permit.approver@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>permit.pco@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>Permit Approver</t>
+  </si>
+  <si>
+    <t>anand.sharma+2023022401@indianic.com/Test@123</t>
+  </si>
+  <si>
+    <t>matt@cybuild.com.au/Commsite12#</t>
+  </si>
+  <si>
+    <t>quoisoforafei-1118@yopmail.com/Test@123</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="@"/>
-  </numFmts>
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -378,22 +373,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -401,7 +381,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <u val="single"/>
+      <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
@@ -418,84 +398,47 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -554,13 +497,26 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -602,12 +558,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -639,7 +595,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -663,7 +619,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -723,42 +679,41 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q35"/>
-  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="22.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="26.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="18.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="21.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="15.14"/>
+    <col min="1" max="1" width="23.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="27" style="1" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="22.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="26.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15" style="1" customWidth="1"/>
+    <col min="13" max="13" width="9" style="1" customWidth="1"/>
+    <col min="14" max="14" width="21.5703125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="41" style="1" customWidth="1"/>
+    <col min="16" max="16" width="17" style="1" customWidth="1"/>
+    <col min="17" max="17" width="15.140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -811,14 +766,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="1">
         <v>14</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -827,7 +782,7 @@
       <c r="E2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="1">
         <v>300000</v>
       </c>
       <c r="G2" s="4" t="s">
@@ -836,7 +791,7 @@
       <c r="H2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="1" t="n">
+      <c r="I2" s="1">
         <v>3600</v>
       </c>
       <c r="J2" s="4" t="s">
@@ -857,27 +812,27 @@
       <c r="O2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="P2" s="1" t="n">
+      <c r="P2" s="1">
         <v>60000</v>
       </c>
       <c r="Q2" s="1" t="str">
-        <f aca="false">Main!B2</f>
+        <f>Main!B2</f>
         <v>UGL</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C3" s="1" t="n">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C3" s="1">
         <v>12</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="1">
         <v>13</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -886,7 +841,7 @@
       <c r="E4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="1">
         <v>300000</v>
       </c>
       <c r="G4" s="4" t="s">
@@ -895,7 +850,7 @@
       <c r="H4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="1" t="n">
+      <c r="I4" s="1">
         <v>3600</v>
       </c>
       <c r="J4" s="4" t="s">
@@ -917,19 +872,19 @@
         <v>23</v>
       </c>
       <c r="P4" s="4"/>
-      <c r="Q4" s="1" t="n">
-        <f aca="false">Main!B4</f>
+      <c r="Q4" s="1">
+        <f>Main!B4</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C6" s="1">
         <v>11</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -938,7 +893,7 @@
       <c r="E6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="F6" s="1">
         <v>300000</v>
       </c>
       <c r="G6" s="4" t="s">
@@ -947,7 +902,7 @@
       <c r="H6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="1" t="n">
+      <c r="I6" s="1">
         <v>3600</v>
       </c>
       <c r="J6" s="4" t="s">
@@ -970,14 +925,14 @@
       </c>
       <c r="P6" s="4"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="C10" s="1">
         <v>13</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -986,7 +941,7 @@
       <c r="E10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="1" t="n">
+      <c r="F10" s="1">
         <v>300000</v>
       </c>
       <c r="G10" s="4" t="s">
@@ -995,7 +950,7 @@
       <c r="H10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I10" s="1" t="n">
+      <c r="I10" s="1">
         <v>3600</v>
       </c>
       <c r="J10" s="4" t="s">
@@ -1018,14 +973,14 @@
       </c>
       <c r="P10" s="4"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="1" t="n">
+      <c r="C14" s="1">
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -1034,7 +989,7 @@
       <c r="E14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F14" s="1" t="n">
+      <c r="F14" s="1">
         <v>300000</v>
       </c>
       <c r="G14" s="4" t="s">
@@ -1043,7 +998,7 @@
       <c r="H14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="1" t="n">
+      <c r="I14" s="1">
         <v>3600</v>
       </c>
       <c r="J14" s="4" t="s">
@@ -1066,14 +1021,14 @@
       </c>
       <c r="P14" s="4"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="1" t="n">
+      <c r="C20" s="1">
         <v>13</v>
       </c>
       <c r="D20" s="1" t="s">
@@ -1082,7 +1037,7 @@
       <c r="E20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F20" s="1" t="n">
+      <c r="F20" s="1">
         <v>300000</v>
       </c>
       <c r="G20" s="4" t="s">
@@ -1091,7 +1046,7 @@
       <c r="H20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I20" s="1" t="n">
+      <c r="I20" s="1">
         <v>3600</v>
       </c>
       <c r="J20" s="4" t="s">
@@ -1114,14 +1069,14 @@
       </c>
       <c r="P20" s="4"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C23" s="1" t="n">
+      <c r="C23" s="1">
         <v>13</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -1130,7 +1085,7 @@
       <c r="E23" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F23" s="1" t="n">
+      <c r="F23" s="1">
         <v>300000</v>
       </c>
       <c r="G23" s="4" t="s">
@@ -1139,7 +1094,7 @@
       <c r="H23" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I23" s="1" t="n">
+      <c r="I23" s="1">
         <v>3600</v>
       </c>
       <c r="J23" s="4" t="s">
@@ -1161,19 +1116,19 @@
         <v>23</v>
       </c>
       <c r="P23" s="4"/>
-      <c r="Q23" s="1" t="n">
-        <f aca="false">Main!B23</f>
+      <c r="Q23" s="1">
+        <f>Main!B23</f>
         <v>0</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="1" t="n">
+      <c r="C25" s="1">
         <v>12</v>
       </c>
       <c r="D25" s="1" t="s">
@@ -1182,7 +1137,7 @@
       <c r="E25" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F25" s="1" t="n">
+      <c r="F25" s="1">
         <v>300000</v>
       </c>
       <c r="G25" s="4" t="s">
@@ -1191,7 +1146,7 @@
       <c r="H25" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I25" s="1" t="n">
+      <c r="I25" s="1">
         <v>3600</v>
       </c>
       <c r="J25" s="4" t="s">
@@ -1214,7 +1169,7 @@
       </c>
       <c r="P25" s="4"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -1230,7 +1185,7 @@
       <c r="E28" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F28" s="1" t="n">
+      <c r="F28" s="1">
         <v>300000</v>
       </c>
       <c r="G28" s="4" t="s">
@@ -1239,7 +1194,7 @@
       <c r="H28" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I28" s="1" t="n">
+      <c r="I28" s="1">
         <v>3600</v>
       </c>
       <c r="J28" s="4" t="s">
@@ -1261,19 +1216,19 @@
         <v>23</v>
       </c>
       <c r="P28" s="4"/>
-      <c r="Q28" s="1" t="n">
-        <f aca="false">Main!B28</f>
+      <c r="Q28" s="1">
+        <f>Main!B28</f>
         <v>0</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="1" t="n">
+      <c r="C33" s="1">
         <v>8</v>
       </c>
       <c r="D33" s="1" t="s">
@@ -1282,7 +1237,7 @@
       <c r="E33" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F33" s="1" t="n">
+      <c r="F33" s="1">
         <v>300000</v>
       </c>
       <c r="G33" s="4" t="s">
@@ -1291,7 +1246,7 @@
       <c r="H33" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I33" s="1" t="n">
+      <c r="I33" s="1">
         <v>3600</v>
       </c>
       <c r="J33" s="4" t="s">
@@ -1313,19 +1268,19 @@
         <v>23</v>
       </c>
       <c r="P33" s="4"/>
-      <c r="Q33" s="1" t="n">
-        <f aca="false">Main!B33</f>
+      <c r="Q33" s="1">
+        <f>Main!B33</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C35" s="1" t="n">
+      <c r="C35" s="1">
         <v>12</v>
       </c>
       <c r="D35" s="1" t="s">
@@ -1334,7 +1289,7 @@
       <c r="E35" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F35" s="1" t="n">
+      <c r="F35" s="1">
         <v>300000</v>
       </c>
       <c r="G35" s="4" t="s">
@@ -1343,7 +1298,7 @@
       <c r="H35" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I35" s="1" t="n">
+      <c r="I35" s="1">
         <v>3600</v>
       </c>
       <c r="J35" s="4" t="s">
@@ -1366,41 +1321,33 @@
       </c>
       <c r="P35" s="4"/>
       <c r="Q35" s="1" t="str">
-        <f aca="false">Main!B35</f>
+        <f>Main!B35</f>
         <v>UGL</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="31.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="30.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="34.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="30.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="46.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.71"/>
+    <col min="1" max="1" width="26.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="34.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="31.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="30.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="34.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="30.42578125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="46.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -1429,45 +1376,45 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
-        <f aca="false">Main!A2</f>
-        <v>https://im-aam.com/</v>
+        <f>Main!A2</f>
+        <v>https://staging.im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
-        <f aca="false">Main!B2</f>
+        <f>Main!B2</f>
         <v>UGL</v>
       </c>
       <c r="C2" s="1" t="str">
-        <f aca="false">Main!D2</f>
+        <f>Main!D2</f>
         <v>anand.sharma+021501@indianic.com/Test@123</v>
       </c>
       <c r="D2" s="1" t="str">
-        <f aca="false">Main!E2</f>
+        <f>Main!E2</f>
         <v>anna.miller@example.com/123456</v>
       </c>
       <c r="E2" s="1" t="str">
-        <f aca="false">Main!F2</f>
+        <f>Main!F2</f>
         <v>qaapprover1.27may2025@yopmail.com/Test@123</v>
       </c>
       <c r="F2" s="1" t="str">
-        <f aca="false">Main!H2</f>
+        <f>Main!H2</f>
         <v>jaydeep.d+040420239@indianic.com/Test@123</v>
       </c>
       <c r="G2" s="1" t="str">
-        <f aca="false">Main!I2</f>
+        <f>Main!I2</f>
         <v>Ad Sd</v>
       </c>
       <c r="H2" s="1" t="str">
-        <f aca="false">Main!J2</f>
+        <f>Main!J2</f>
         <v>coUser1.15july2025@yopmail.com/Test@123</v>
       </c>
       <c r="I2" s="1" t="str">
-        <f aca="false">Main!O2</f>
+        <f>Main!O2</f>
         <v>E&amp;IC</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>37</v>
       </c>
@@ -1490,7 +1437,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C13" s="1" t="s">
         <v>44</v>
       </c>
@@ -1506,43 +1453,35 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A11" r:id="rId1" display="http://cybuild.devpress.net"/>
+    <hyperlink ref="A11" r:id="rId1"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O13"/>
-  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="44.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="32.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="47.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="48.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="43.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="25.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="40.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="42.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="41.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="46.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="35.57"/>
+    <col min="1" max="1" width="30.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16" style="1" customWidth="1"/>
+    <col min="4" max="4" width="44.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="32.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="47.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="48.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="43.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="25.7109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="40.140625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="42.85546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="41.28515625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="46.7109375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="35.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -1589,69 +1528,69 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
-        <f aca="false">Main!A2</f>
-        <v>https://im-aam.com/</v>
+        <f>Main!A2</f>
+        <v>https://staging.im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
-        <f aca="false">Main!B2</f>
+        <f>Main!B2</f>
         <v>UGL</v>
       </c>
       <c r="C2" s="1" t="str">
-        <f aca="false">Main!C2</f>
+        <f>Main!C2</f>
         <v>Hunter Power Project</v>
       </c>
       <c r="D2" s="1" t="str">
-        <f aca="false">Main!D2</f>
+        <f>Main!D2</f>
         <v>anand.sharma+021501@indianic.com/Test@123</v>
       </c>
       <c r="E2" s="1" t="str">
-        <f aca="false">Main!E2</f>
+        <f>Main!E2</f>
         <v>anna.miller@example.com/123456</v>
       </c>
       <c r="F2" s="1" t="str">
-        <f aca="false">Main!F2</f>
+        <f>Main!F2</f>
         <v>qaapprover1.27may2025@yopmail.com/Test@123</v>
       </c>
       <c r="G2" s="1" t="str">
-        <f aca="false">Main!G2</f>
+        <f>Main!G2</f>
         <v>qaapprover2.27may2025@yopmail.com/Test@123</v>
       </c>
       <c r="H2" s="1" t="str">
-        <f aca="false">Main!H2</f>
+        <f>Main!H2</f>
         <v>jaydeep.d+040420239@indianic.com/Test@123</v>
       </c>
       <c r="I2" s="1" t="str">
-        <f aca="false">Main!I2</f>
+        <f>Main!I2</f>
         <v>Ad Sd</v>
       </c>
       <c r="J2" s="1" t="str">
-        <f aca="false">Main!J2</f>
+        <f>Main!J2</f>
         <v>coUser1.15july2025@yopmail.com/Test@123</v>
       </c>
       <c r="K2" s="1" t="str">
-        <f aca="false">Main!K2</f>
+        <f>Main!K2</f>
         <v>supervisor.27may2025@yopmail.com/Test@123</v>
       </c>
       <c r="L2" s="1" t="str">
-        <f aca="false">Main!L2</f>
+        <f>Main!L2</f>
         <v>engineer.27may2025@yopmail.com/Test@123</v>
       </c>
       <c r="M2" s="1" t="str">
-        <f aca="false">Main!M2</f>
+        <f>Main!M2</f>
         <v>technicaladmin.27may2025@yopmail.com/Test@123</v>
       </c>
       <c r="N2" s="1" t="str">
-        <f aca="false">Main!N2</f>
+        <f>Main!N2</f>
         <v>admin@cybuild.com.au/Commsite12#</v>
       </c>
       <c r="O2" s="1" t="str">
-        <f aca="false">Main!O2</f>
+        <f>Main!O2</f>
         <v>E&amp;IC</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>37</v>
       </c>
@@ -1675,7 +1614,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D13" s="1" t="s">
         <v>44</v>
       </c>
@@ -1691,43 +1630,35 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A11" r:id="rId1" display="http://cybuild.devpress.net"/>
+    <hyperlink ref="A11" r:id="rId1"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O49"/>
-  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="48.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="47.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="43.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="48.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="41.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="47.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="35.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="10.57"/>
+    <col min="1" max="1" width="30.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="48.42578125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="41.42578125" style="1" customWidth="1"/>
+    <col min="6" max="7" width="47.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="43.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="30.42578125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="48.140625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="43" style="1" customWidth="1"/>
+    <col min="12" max="12" width="41.7109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="47.28515625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="35.5703125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="10.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -1774,9 +1705,9 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>55</v>
@@ -1821,7 +1752,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>69</v>
       </c>
@@ -1832,12 +1763,12 @@
         <v>71</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>72</v>
       </c>
@@ -1860,7 +1791,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>73</v>
       </c>
@@ -1883,7 +1814,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>73</v>
       </c>
@@ -1906,7 +1837,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>73</v>
       </c>
@@ -1929,7 +1860,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D17" s="1" t="s">
         <v>39</v>
       </c>
@@ -1940,7 +1871,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F18" s="1" t="s">
         <v>88</v>
       </c>
@@ -1951,13 +1882,13 @@
         <v>43</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B19" s="5"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>73</v>
       </c>
@@ -1980,7 +1911,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>73</v>
       </c>
@@ -2006,7 +1937,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>72</v>
       </c>
@@ -2038,22 +1969,22 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C32" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>100</v>
       </c>
@@ -2085,7 +2016,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
         <v>55</v>
       </c>
@@ -2093,7 +2024,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>104</v>
       </c>
@@ -2125,12 +2056,12 @@
         <v>67</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C41" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>100</v>
       </c>
@@ -2165,7 +2096,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>100</v>
       </c>
@@ -2200,7 +2131,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>98</v>
       </c>
@@ -2247,50 +2178,45 @@
         <v>68</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J49" s="1" t="s">
         <v>110</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" display="anna.miller@example.com/123456"/>
-    <hyperlink ref="K2" r:id="rId2" display="supervisor.27may2025@yopmail.com/Test@123"/>
-    <hyperlink ref="L2" r:id="rId3" display="engineer.27may2025@yopmail.com/Test@123"/>
-    <hyperlink ref="M2" r:id="rId4" display="technicaladmin.27may2025@yopmail.com/Test@123"/>
-    <hyperlink ref="J4" r:id="rId5" display="matt@acompletions.com/123456"/>
-    <hyperlink ref="J6" r:id="rId6" display="dhaval.barot@indianic.com/123456"/>
-    <hyperlink ref="F12" r:id="rId7" display="987789654/Test@123"/>
-    <hyperlink ref="F14" r:id="rId8" display="test02152023120271@yopmail.com/Test@123"/>
-    <hyperlink ref="H14" r:id="rId9" display="test021520231202899@yopmail.com/Test@123"/>
-    <hyperlink ref="J14" r:id="rId10" display="matt@acompletions.com/123456"/>
-    <hyperlink ref="J18" r:id="rId11" display="dhaval.barot@indianic.com/123456"/>
-    <hyperlink ref="D24" r:id="rId12" display="1May2023-l2@yopmail.com/Test@123"/>
-    <hyperlink ref="F24" r:id="rId13" display="1May2023-l4@yopmail.com/Test@123"/>
-    <hyperlink ref="H24" r:id="rId14" display="1May2023-pco@yopmail.com/Test@123"/>
-    <hyperlink ref="J24" r:id="rId15" display="matt@acompletions.com/123456"/>
-    <hyperlink ref="A26" r:id="rId16" display="https://dev.cybuild.com.au/"/>
-    <hyperlink ref="E26" r:id="rId17" display="anna.miller@example.com/123456"/>
-    <hyperlink ref="J26" r:id="rId18" display="matt@acompletions.com/123456"/>
-    <hyperlink ref="A28" r:id="rId19" display="https://dev.cybuild.com.au/"/>
-    <hyperlink ref="E34" r:id="rId20" display="anna.miller@example.com/123456"/>
-    <hyperlink ref="J34" r:id="rId21" display="matt@acompletions.com/123456"/>
-    <hyperlink ref="E37" r:id="rId22" display="anna.miller@example.com/123456"/>
-    <hyperlink ref="J37" r:id="rId23" display="matt@acompletions.com/123456"/>
-    <hyperlink ref="E43" r:id="rId24" display="anna.miller@example.com/123456"/>
-    <hyperlink ref="J43" r:id="rId25" display="matt@acompletions.com/123456"/>
-    <hyperlink ref="E46" r:id="rId26" display="anna.miller@example.com/123456"/>
-    <hyperlink ref="E48" r:id="rId27" display="anna.miller@example.com/123456"/>
-    <hyperlink ref="K48" r:id="rId28" display="supervisor.27may2025@yopmail.com/Test@123"/>
-    <hyperlink ref="L48" r:id="rId29" display="engineer.27may2025@yopmail.com/Test@123"/>
-    <hyperlink ref="M48" r:id="rId30" display="technicaladmin.27may2025@yopmail.com/Test@123"/>
+    <hyperlink ref="E2" r:id="rId1"/>
+    <hyperlink ref="K2" r:id="rId2"/>
+    <hyperlink ref="L2" r:id="rId3"/>
+    <hyperlink ref="M2" r:id="rId4"/>
+    <hyperlink ref="J4" r:id="rId5"/>
+    <hyperlink ref="J6" r:id="rId6"/>
+    <hyperlink ref="F12" r:id="rId7"/>
+    <hyperlink ref="F14" r:id="rId8"/>
+    <hyperlink ref="H14" r:id="rId9"/>
+    <hyperlink ref="J14" r:id="rId10"/>
+    <hyperlink ref="J18" r:id="rId11"/>
+    <hyperlink ref="D24" r:id="rId12"/>
+    <hyperlink ref="F24" r:id="rId13"/>
+    <hyperlink ref="H24" r:id="rId14"/>
+    <hyperlink ref="J24" r:id="rId15"/>
+    <hyperlink ref="A26" r:id="rId16"/>
+    <hyperlink ref="E26" r:id="rId17"/>
+    <hyperlink ref="J26" r:id="rId18"/>
+    <hyperlink ref="A28" r:id="rId19"/>
+    <hyperlink ref="E34" r:id="rId20"/>
+    <hyperlink ref="J34" r:id="rId21"/>
+    <hyperlink ref="E37" r:id="rId22"/>
+    <hyperlink ref="J37" r:id="rId23"/>
+    <hyperlink ref="E43" r:id="rId24"/>
+    <hyperlink ref="J43" r:id="rId25"/>
+    <hyperlink ref="E46" r:id="rId26"/>
+    <hyperlink ref="E48" r:id="rId27"/>
+    <hyperlink ref="K48" r:id="rId28"/>
+    <hyperlink ref="L48" r:id="rId29"/>
+    <hyperlink ref="M48" r:id="rId30"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Latest changes on 23Aug2026
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -1379,7 +1379,7 @@
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://staging.im-aam.com/</v>
+        <v>https://im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1531,7 +1531,7 @@
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://staging.im-aam.com/</v>
+        <v>https://im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1707,7 +1707,7 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Latest changes on 24August2026.
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -1379,7 +1379,7 @@
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://im-aam.com/</v>
+        <v>https://staging.im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1531,7 +1531,7 @@
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://im-aam.com/</v>
+        <v>https://staging.im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1707,7 +1707,7 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Latest changes on 28Aug2026
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -1379,7 +1379,7 @@
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://staging.im-aam.com/</v>
+        <v>https://im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1531,7 +1531,7 @@
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://staging.im-aam.com/</v>
+        <v>https://im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1707,7 +1707,7 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Latest changes on 29Aug2026
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -1379,7 +1379,7 @@
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://im-aam.com/</v>
+        <v>https://staging.im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1531,7 +1531,7 @@
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://im-aam.com/</v>
+        <v>https://staging.im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1707,7 +1707,7 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Latest changes on 30 Aug 2026
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -1379,7 +1379,7 @@
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://staging.im-aam.com/</v>
+        <v>https://im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1531,7 +1531,7 @@
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://staging.im-aam.com/</v>
+        <v>https://im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1707,7 +1707,7 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Latest changes on 31 Aug 2026
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -1379,7 +1379,7 @@
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://im-aam.com/</v>
+        <v>https://staging.im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1531,7 +1531,7 @@
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://im-aam.com/</v>
+        <v>https://staging.im-aam.com/</v>
       </c>
       <c r="B2" s="1" t="str">
         <f>Main!B2</f>
@@ -1707,7 +1707,7 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Latest changes on 8Sept2026.
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="61">
   <si>
     <t>Device Name</t>
   </si>
@@ -189,36 +189,6 @@
     <t>https://im-aam.com/</t>
   </si>
   <si>
-    <t>UGL</t>
-  </si>
-  <si>
-    <t>Hunter Power Project</t>
-  </si>
-  <si>
-    <t>anand.sharma+021501@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>anna.miller@example.com/123456</t>
-  </si>
-  <si>
-    <t>qaapprover1.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>qaapprover2.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>jaydeep.d+040420239@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>Ad Sd</t>
-  </si>
-  <si>
-    <t>coUser1.15july2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>supervisor.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
     <t>engineer.27may2025@yopmail.com/Test@123</t>
   </si>
   <si>
@@ -234,130 +204,7 @@
     <t>https://staging.im-aam.com/</t>
   </si>
   <si>
-    <t>hiren.joshi+L201PH@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>matt@acompletions.com/123456</t>
-  </si>
-  <si>
-    <t>https://dev.cybuild.com.au/</t>
-  </si>
-  <si>
-    <t>https://cybuild.com.au</t>
-  </si>
-  <si>
-    <t>Demo Project</t>
-  </si>
-  <si>
-    <t>hiren.joshi+L401PA@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>hiren.joshi+L701PCO@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>HirenEdited Joshi L4 01 PAEdited</t>
-  </si>
-  <si>
-    <t>anand.sharma+20230501@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>987671231/Test@123</t>
-  </si>
-  <si>
-    <t>987789654/Test@123</t>
-  </si>
-  <si>
-    <t>789123321/Test@123</t>
-  </si>
-  <si>
-    <t>15feb-1@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>test02152023120271@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>test021520231202899@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>L4 User</t>
-  </si>
-  <si>
-    <t>qaapprover3@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>qaapprover4@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>qaapprover1@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>qaapprover2@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>https://cybuild.devpress.net</t>
-  </si>
-  <si>
-    <t>permitwriter@example.com/Test@123</t>
-  </si>
-  <si>
-    <t>1May2023-l2@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>1May2023-l4@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>1May2023-pco@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>1May2023 L4</t>
-  </si>
-  <si>
     <t>acompletions@admin.com/123456</t>
-  </si>
-  <si>
-    <t>sara.johansen@example.com/123456</t>
-  </si>
-  <si>
-    <t>https://dev-ugl.cybuild.com.au/</t>
-  </si>
-  <si>
-    <t>Work Pack Demo</t>
-  </si>
-  <si>
-    <t>https://dev-app.cybuild.com.au/</t>
-  </si>
-  <si>
-    <t>John Holland</t>
-  </si>
-  <si>
-    <t>WestConnex 3B</t>
-  </si>
-  <si>
-    <t>anand.sharma+040420232@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>https://app.cybuild.com.au</t>
-  </si>
-  <si>
-    <t>permit.writer@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>permit.approver@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>permit.pco@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>Permit Approver</t>
-  </si>
-  <si>
-    <t>anand.sharma+2023022401@indianic.com/Test@123</t>
-  </si>
-  <si>
-    <t>matt@cybuild.com.au/Commsite12#</t>
-  </si>
-  <si>
-    <t>quoisoforafei-1118@yopmail.com/Test@123</t>
   </si>
 </sst>
 </file>
@@ -815,9 +662,9 @@
       <c r="P2" s="1">
         <v>60000</v>
       </c>
-      <c r="Q2" s="1" t="str">
+      <c r="Q2" s="1">
         <f>Main!B2</f>
-        <v>UGL</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -1320,9 +1167,9 @@
         <v>23</v>
       </c>
       <c r="P35" s="4"/>
-      <c r="Q35" s="1" t="str">
+      <c r="Q35" s="1">
         <f>Main!B35</f>
-        <v>UGL</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1379,39 +1226,39 @@
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://staging.im-aam.com/</v>
-      </c>
-      <c r="B2" s="1" t="str">
+        <v>https://im-aam.com/</v>
+      </c>
+      <c r="B2" s="1">
         <f>Main!B2</f>
-        <v>UGL</v>
-      </c>
-      <c r="C2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1">
         <f>Main!D2</f>
-        <v>anand.sharma+021501@indianic.com/Test@123</v>
-      </c>
-      <c r="D2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1">
         <f>Main!E2</f>
-        <v>anna.miller@example.com/123456</v>
-      </c>
-      <c r="E2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
         <f>Main!F2</f>
-        <v>qaapprover1.27may2025@yopmail.com/Test@123</v>
-      </c>
-      <c r="F2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
         <f>Main!H2</f>
-        <v>jaydeep.d+040420239@indianic.com/Test@123</v>
-      </c>
-      <c r="G2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
         <f>Main!I2</f>
-        <v>Ad Sd</v>
-      </c>
-      <c r="H2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
         <f>Main!J2</f>
-        <v>coUser1.15july2025@yopmail.com/Test@123</v>
-      </c>
-      <c r="I2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1">
         <f>Main!O2</f>
-        <v>E&amp;IC</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -1531,63 +1378,63 @@
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>Main!A2</f>
-        <v>https://staging.im-aam.com/</v>
-      </c>
-      <c r="B2" s="1" t="str">
+        <v>https://im-aam.com/</v>
+      </c>
+      <c r="B2" s="1">
         <f>Main!B2</f>
-        <v>UGL</v>
-      </c>
-      <c r="C2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1">
         <f>Main!C2</f>
-        <v>Hunter Power Project</v>
-      </c>
-      <c r="D2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1">
         <f>Main!D2</f>
-        <v>anand.sharma+021501@indianic.com/Test@123</v>
-      </c>
-      <c r="E2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
         <f>Main!E2</f>
-        <v>anna.miller@example.com/123456</v>
-      </c>
-      <c r="F2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
         <f>Main!F2</f>
-        <v>qaapprover1.27may2025@yopmail.com/Test@123</v>
-      </c>
-      <c r="G2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
         <f>Main!G2</f>
-        <v>qaapprover2.27may2025@yopmail.com/Test@123</v>
-      </c>
-      <c r="H2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
         <f>Main!H2</f>
-        <v>jaydeep.d+040420239@indianic.com/Test@123</v>
-      </c>
-      <c r="I2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1">
         <f>Main!I2</f>
-        <v>Ad Sd</v>
-      </c>
-      <c r="J2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1">
         <f>Main!J2</f>
-        <v>coUser1.15july2025@yopmail.com/Test@123</v>
-      </c>
-      <c r="K2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1">
         <f>Main!K2</f>
-        <v>supervisor.27may2025@yopmail.com/Test@123</v>
-      </c>
-      <c r="L2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="L2" s="1">
         <f>Main!L2</f>
-        <v>engineer.27may2025@yopmail.com/Test@123</v>
-      </c>
-      <c r="M2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="M2" s="1">
         <f>Main!M2</f>
-        <v>technicaladmin.27may2025@yopmail.com/Test@123</v>
-      </c>
-      <c r="N2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="N2" s="1">
         <f>Main!N2</f>
-        <v>admin@cybuild.com.au/Commsite12#</v>
-      </c>
-      <c r="O2" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="O2" s="1">
         <f>Main!O2</f>
-        <v>E&amp;IC</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -1639,7 +1486,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.140625" style="1" customWidth="1"/>
@@ -1707,60 +1554,12 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1768,453 +1567,62 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="D17" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F18" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>90</v>
-      </c>
+    <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B19" s="5"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>71</v>
-      </c>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N24" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B26" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="N26" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="34" spans="12:15" x14ac:dyDescent="0.25">
+      <c r="N34" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="37" spans="12:15" x14ac:dyDescent="0.25">
+      <c r="N37" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="43" spans="12:15" x14ac:dyDescent="0.25">
+      <c r="N43" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="46" spans="12:15" x14ac:dyDescent="0.25">
+      <c r="N46" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="48" spans="12:15" x14ac:dyDescent="0.25">
+      <c r="L48" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="M48" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E26" s="1" t="s">
+      <c r="N48" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="O48" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="N26" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C32" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="N34" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="H37" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="I37" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="N37" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C41" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="H43" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I43" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="N43" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="H46" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I46" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="J46" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="N46" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F48" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G48" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="H48" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I48" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="J48" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="K48" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="L48" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="M48" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="N48" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="O48" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="49" spans="10:10" x14ac:dyDescent="0.25">
-      <c r="J49" s="1" t="s">
-        <v>110</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1"/>
-    <hyperlink ref="K2" r:id="rId2"/>
-    <hyperlink ref="L2" r:id="rId3"/>
-    <hyperlink ref="M2" r:id="rId4"/>
-    <hyperlink ref="J4" r:id="rId5"/>
-    <hyperlink ref="J6" r:id="rId6"/>
-    <hyperlink ref="F12" r:id="rId7"/>
-    <hyperlink ref="F14" r:id="rId8"/>
-    <hyperlink ref="H14" r:id="rId9"/>
-    <hyperlink ref="J14" r:id="rId10"/>
-    <hyperlink ref="J18" r:id="rId11"/>
-    <hyperlink ref="D24" r:id="rId12"/>
-    <hyperlink ref="F24" r:id="rId13"/>
-    <hyperlink ref="H24" r:id="rId14"/>
-    <hyperlink ref="J24" r:id="rId15"/>
-    <hyperlink ref="A26" r:id="rId16"/>
-    <hyperlink ref="E26" r:id="rId17"/>
-    <hyperlink ref="J26" r:id="rId18"/>
-    <hyperlink ref="A28" r:id="rId19"/>
-    <hyperlink ref="E34" r:id="rId20"/>
-    <hyperlink ref="J34" r:id="rId21"/>
-    <hyperlink ref="E37" r:id="rId22"/>
-    <hyperlink ref="J37" r:id="rId23"/>
-    <hyperlink ref="E43" r:id="rId24"/>
-    <hyperlink ref="J43" r:id="rId25"/>
-    <hyperlink ref="E46" r:id="rId26"/>
-    <hyperlink ref="E48" r:id="rId27"/>
-    <hyperlink ref="K48" r:id="rId28"/>
-    <hyperlink ref="L48" r:id="rId29"/>
-    <hyperlink ref="M48" r:id="rId30"/>
+    <hyperlink ref="L48" r:id="rId1"/>
+    <hyperlink ref="M48" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Latest changes on 9Sept2026
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="5"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
-    <sheet name="configMobile" sheetId="1" r:id="rId1"/>
-    <sheet name="permitFlow" sheetId="2" r:id="rId2"/>
-    <sheet name="testFlow" sheetId="3" r:id="rId3"/>
-    <sheet name="Main" sheetId="4" r:id="rId4"/>
+    <sheet name="configMobile" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="permitFlow" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="testFlow" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Main" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="144525" iterateDelta="1E-4"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -24,194 +25,198 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="61">
   <si>
-    <t>Device Name</t>
-  </si>
-  <si>
-    <t>Platform Name</t>
-  </si>
-  <si>
-    <t>Platform Version</t>
-  </si>
-  <si>
-    <t>Automation Name</t>
-  </si>
-  <si>
-    <t>Skip Unlock</t>
-  </si>
-  <si>
-    <t>AVD Launch Timeout</t>
-  </si>
-  <si>
-    <t>Ensure Webview Have Pages</t>
-  </si>
-  <si>
-    <t>Native Web Screenshot</t>
-  </si>
-  <si>
-    <t>New Command Timeout</t>
-  </si>
-  <si>
-    <t>Connect Hardware Keyboard</t>
-  </si>
-  <si>
-    <t>Unicoded Keyboard</t>
-  </si>
-  <si>
-    <t>Reset Keyboard</t>
-  </si>
-  <si>
-    <t>No Reset</t>
-  </si>
-  <si>
-    <t>App Package</t>
-  </si>
-  <si>
-    <t>App Activity</t>
-  </si>
-  <si>
-    <t>Adb Exec Timeout</t>
-  </si>
-  <si>
-    <t>Client Company</t>
-  </si>
-  <si>
-    <t>sdk_gphone64_x86_64</t>
-  </si>
-  <si>
-    <t>Android</t>
-  </si>
-  <si>
-    <t>UiAutomator2</t>
-  </si>
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>false</t>
-  </si>
-  <si>
-    <t>com.app.acompletions</t>
-  </si>
-  <si>
-    <t>com.commissioning.ui.splash.SplashActivity</t>
-  </si>
-  <si>
-    <t>Android SDK built for x86</t>
-  </si>
-  <si>
-    <t>Pixel C</t>
-  </si>
-  <si>
-    <t>Redmi26</t>
-  </si>
-  <si>
-    <t>8.1.0</t>
-  </si>
-  <si>
-    <t>Environment URL</t>
-  </si>
-  <si>
-    <t>Project Name</t>
-  </si>
-  <si>
-    <t>L2 User Credentials</t>
-  </si>
-  <si>
-    <t>Permit Holder Credentials</t>
-  </si>
-  <si>
-    <t>L4 User Credentials</t>
-  </si>
-  <si>
-    <t>PCO User Credentials</t>
-  </si>
-  <si>
-    <t>Permit Approver (L4) Name</t>
-  </si>
-  <si>
-    <t>Projectr Admin Credentials</t>
-  </si>
-  <si>
-    <t>Discipline</t>
-  </si>
-  <si>
-    <t>http://cybuild.devpress.net</t>
-  </si>
-  <si>
-    <t>Brave</t>
-  </si>
-  <si>
-    <t>todd.beck@example.com/123456</t>
-  </si>
-  <si>
-    <t>julie.cole@example.com/123456</t>
-  </si>
-  <si>
-    <t>noah.poulsen@example.com/123456</t>
-  </si>
-  <si>
-    <t>Julie Cole</t>
-  </si>
-  <si>
-    <t>dhaval.barot@indianic.com/123456</t>
-  </si>
-  <si>
-    <t>tom@mac-24.com/Test@123</t>
-  </si>
-  <si>
-    <t>john@mac-24.com/123456</t>
-  </si>
-  <si>
-    <t>kevin@mac-24.com/123456</t>
-  </si>
-  <si>
-    <t>Niall Stenson</t>
-  </si>
-  <si>
-    <t>QA Manager Credentials</t>
-  </si>
-  <si>
-    <t>Project Admin Credentials</t>
-  </si>
-  <si>
-    <t>Supervisor Credentials</t>
-  </si>
-  <si>
-    <t>Engineer Credentials</t>
-  </si>
-  <si>
-    <t>Technical Admin Credentials</t>
-  </si>
-  <si>
-    <t>Super Admin Credentials</t>
-  </si>
-  <si>
-    <t>https://im-aam.com/</t>
-  </si>
-  <si>
-    <t>engineer.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>technicaladmin.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t>admin@cybuild.com.au/Commsite12#</t>
-  </si>
-  <si>
-    <t>E&amp;IC</t>
-  </si>
-  <si>
-    <t>https://staging.im-aam.com/</t>
-  </si>
-  <si>
-    <t>acompletions@admin.com/123456</t>
+    <t xml:space="preserve">Device Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Platform Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Platform Version</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automation Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skip Unlock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVD Launch Timeout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ensure Webview Have Pages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Native Web Screenshot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New Command Timeout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Connect Hardware Keyboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unicoded Keyboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reset Keyboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Reset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App Package</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App Activity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adb Exec Timeout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Client Company</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdk_gphone64_x86_64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Android</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UiAutomator2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">true</t>
+  </si>
+  <si>
+    <t xml:space="preserve">false</t>
+  </si>
+  <si>
+    <t xml:space="preserve">com.app.acompletions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">com.commissioning.ui.splash.SplashActivity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Android SDK built for x86</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pixel C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redmi26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.1.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Environment URL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L2 User Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit Holder Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L4 User Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCO User Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit Approver (L4) Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projectr Admin Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discipline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://cybuild.devpress.net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brave</t>
+  </si>
+  <si>
+    <t xml:space="preserve">todd.beck@example.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">julie.cole@example.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">noah.poulsen@example.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Julie Cole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dhaval.barot@indianic.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tom@mac-24.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">john@mac-24.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kevin@mac-24.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niall Stenson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QA Manager Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project Admin Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supervisor Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engineer Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technical Admin Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Admin Credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://im-aam.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://staging.im-aam.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">acompletions@admin.com/123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">admin@cybuild.com.au/Commsite12#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">engineer.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">technicaladmin.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E&amp;IC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="@"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -220,7 +225,22 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -228,7 +248,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <u/>
+      <u val="single"/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
@@ -245,47 +265,84 @@
     </fill>
   </fills>
   <borders count="2">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+  <cellStyleXfs count="21">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -344,26 +401,13 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -405,12 +449,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Calibri Light" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -442,7 +486,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -466,7 +510,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -526,41 +570,42 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:Q35"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="23.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="27" style="1" customWidth="1"/>
-    <col min="8" max="8" width="22.28515625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="22.85546875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26.7109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="18.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15" style="1" customWidth="1"/>
-    <col min="13" max="13" width="9" style="1" customWidth="1"/>
-    <col min="14" max="14" width="21.5703125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="41" style="1" customWidth="1"/>
-    <col min="16" max="16" width="17" style="1" customWidth="1"/>
-    <col min="17" max="17" width="15.140625" style="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="22.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="26.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="18.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="21.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="15.14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -613,14 +658,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="1" t="n">
         <v>14</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -629,7 +674,7 @@
       <c r="E2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G2" s="4" t="s">
@@ -638,7 +683,7 @@
       <c r="H2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J2" s="4" t="s">
@@ -659,27 +704,27 @@
       <c r="O2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="1" t="n">
         <v>60000</v>
       </c>
-      <c r="Q2" s="1">
-        <f>Main!B2</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C3" s="1">
+      <c r="Q2" s="1" t="n">
+        <f aca="false">Main!B2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C3" s="1" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="1" t="n">
         <v>13</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -688,7 +733,7 @@
       <c r="E4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G4" s="4" t="s">
@@ -697,7 +742,7 @@
       <c r="H4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J4" s="4" t="s">
@@ -719,19 +764,19 @@
         <v>23</v>
       </c>
       <c r="P4" s="4"/>
-      <c r="Q4" s="1">
-        <f>Main!B4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q4" s="1" t="n">
+        <f aca="false">Main!B4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="1" t="n">
         <v>11</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -740,7 +785,7 @@
       <c r="E6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G6" s="4" t="s">
@@ -749,7 +794,7 @@
       <c r="H6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J6" s="4" t="s">
@@ -772,14 +817,14 @@
       </c>
       <c r="P6" s="4"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="1" t="n">
         <v>13</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -788,7 +833,7 @@
       <c r="E10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G10" s="4" t="s">
@@ -797,7 +842,7 @@
       <c r="H10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J10" s="4" t="s">
@@ -820,14 +865,14 @@
       </c>
       <c r="P10" s="4"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="1" t="n">
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -836,7 +881,7 @@
       <c r="E14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F14" s="1">
+      <c r="F14" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G14" s="4" t="s">
@@ -845,7 +890,7 @@
       <c r="H14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J14" s="4" t="s">
@@ -868,14 +913,14 @@
       </c>
       <c r="P14" s="4"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="1" t="n">
         <v>13</v>
       </c>
       <c r="D20" s="1" t="s">
@@ -884,7 +929,7 @@
       <c r="E20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F20" s="1">
+      <c r="F20" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G20" s="4" t="s">
@@ -893,7 +938,7 @@
       <c r="H20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I20" s="1">
+      <c r="I20" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J20" s="4" t="s">
@@ -916,14 +961,14 @@
       </c>
       <c r="P20" s="4"/>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C23" s="1">
+      <c r="C23" s="1" t="n">
         <v>13</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -932,7 +977,7 @@
       <c r="E23" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F23" s="1">
+      <c r="F23" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G23" s="4" t="s">
@@ -941,7 +986,7 @@
       <c r="H23" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I23" s="1">
+      <c r="I23" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J23" s="4" t="s">
@@ -963,19 +1008,19 @@
         <v>23</v>
       </c>
       <c r="P23" s="4"/>
-      <c r="Q23" s="1">
-        <f>Main!B23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q23" s="1" t="n">
+        <f aca="false">Main!B23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25" s="1" t="n">
         <v>12</v>
       </c>
       <c r="D25" s="1" t="s">
@@ -984,7 +1029,7 @@
       <c r="E25" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F25" s="1">
+      <c r="F25" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G25" s="4" t="s">
@@ -993,7 +1038,7 @@
       <c r="H25" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I25" s="1">
+      <c r="I25" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J25" s="4" t="s">
@@ -1016,7 +1061,7 @@
       </c>
       <c r="P25" s="4"/>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -1032,7 +1077,7 @@
       <c r="E28" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F28" s="1">
+      <c r="F28" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G28" s="4" t="s">
@@ -1041,7 +1086,7 @@
       <c r="H28" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I28" s="1">
+      <c r="I28" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J28" s="4" t="s">
@@ -1063,19 +1108,19 @@
         <v>23</v>
       </c>
       <c r="P28" s="4"/>
-      <c r="Q28" s="1">
-        <f>Main!B28</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q28" s="1" t="n">
+        <f aca="false">Main!B28</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="1">
+      <c r="C33" s="1" t="n">
         <v>8</v>
       </c>
       <c r="D33" s="1" t="s">
@@ -1084,7 +1129,7 @@
       <c r="E33" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F33" s="1">
+      <c r="F33" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G33" s="4" t="s">
@@ -1093,7 +1138,7 @@
       <c r="H33" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I33" s="1">
+      <c r="I33" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J33" s="4" t="s">
@@ -1115,19 +1160,19 @@
         <v>23</v>
       </c>
       <c r="P33" s="4"/>
-      <c r="Q33" s="1">
-        <f>Main!B33</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q33" s="1" t="n">
+        <f aca="false">Main!B33</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C35" s="1">
+      <c r="C35" s="1" t="n">
         <v>12</v>
       </c>
       <c r="D35" s="1" t="s">
@@ -1136,7 +1181,7 @@
       <c r="E35" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F35" s="1">
+      <c r="F35" s="1" t="n">
         <v>300000</v>
       </c>
       <c r="G35" s="4" t="s">
@@ -1145,7 +1190,7 @@
       <c r="H35" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I35" s="1">
+      <c r="I35" s="1" t="n">
         <v>3600</v>
       </c>
       <c r="J35" s="4" t="s">
@@ -1167,34 +1212,42 @@
         <v>23</v>
       </c>
       <c r="P35" s="4"/>
-      <c r="Q35" s="1">
-        <f>Main!B35</f>
+      <c r="Q35" s="1" t="n">
+        <f aca="false">Main!B35</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="26.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="34.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="31.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="30.7109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="34.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="30.42578125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="46.28515625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" style="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="31.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="30.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="34.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="30.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="46.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.71"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -1223,45 +1276,45 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="str">
-        <f>Main!A2</f>
+        <f aca="false">Main!A2</f>
         <v>https://im-aam.com/</v>
       </c>
-      <c r="B2" s="1">
-        <f>Main!B2</f>
-        <v>0</v>
-      </c>
-      <c r="C2" s="1">
-        <f>Main!D2</f>
-        <v>0</v>
-      </c>
-      <c r="D2" s="1">
-        <f>Main!E2</f>
-        <v>0</v>
-      </c>
-      <c r="E2" s="1">
-        <f>Main!F2</f>
-        <v>0</v>
-      </c>
-      <c r="F2" s="1">
-        <f>Main!H2</f>
-        <v>0</v>
-      </c>
-      <c r="G2" s="1">
-        <f>Main!I2</f>
-        <v>0</v>
-      </c>
-      <c r="H2" s="1">
-        <f>Main!J2</f>
-        <v>0</v>
-      </c>
-      <c r="I2" s="1">
-        <f>Main!O2</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="n">
+        <f aca="false">Main!B2</f>
+        <v>0</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <f aca="false">Main!D2</f>
+        <v>0</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <f aca="false">Main!E2</f>
+        <v>0</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <f aca="false">Main!F2</f>
+        <v>0</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <f aca="false">Main!H2</f>
+        <v>0</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <f aca="false">Main!I2</f>
+        <v>0</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <f aca="false">Main!J2</f>
+        <v>0</v>
+      </c>
+      <c r="I2" s="1" t="n">
+        <f aca="false">Main!O2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>37</v>
       </c>
@@ -1284,7 +1337,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C13" s="1" t="s">
         <v>44</v>
       </c>
@@ -1300,35 +1353,43 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A11" r:id="rId1"/>
+    <hyperlink ref="A11" r:id="rId1" display="http://cybuild.devpress.net"/>
   </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:O13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16" style="1" customWidth="1"/>
-    <col min="4" max="4" width="44.140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="32.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="47.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="48.28515625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="43.5703125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="25.7109375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="40.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="42.85546875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="41.28515625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="46.7109375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="35.5703125" style="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="44.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="32.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="47.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="48.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="43.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="25.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="40.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="42.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="41.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="46.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="35.57"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -1375,69 +1436,69 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="str">
-        <f>Main!A2</f>
+        <f aca="false">Main!A2</f>
         <v>https://im-aam.com/</v>
       </c>
-      <c r="B2" s="1">
-        <f>Main!B2</f>
-        <v>0</v>
-      </c>
-      <c r="C2" s="1">
-        <f>Main!C2</f>
-        <v>0</v>
-      </c>
-      <c r="D2" s="1">
-        <f>Main!D2</f>
-        <v>0</v>
-      </c>
-      <c r="E2" s="1">
-        <f>Main!E2</f>
-        <v>0</v>
-      </c>
-      <c r="F2" s="1">
-        <f>Main!F2</f>
-        <v>0</v>
-      </c>
-      <c r="G2" s="1">
-        <f>Main!G2</f>
-        <v>0</v>
-      </c>
-      <c r="H2" s="1">
-        <f>Main!H2</f>
-        <v>0</v>
-      </c>
-      <c r="I2" s="1">
-        <f>Main!I2</f>
-        <v>0</v>
-      </c>
-      <c r="J2" s="1">
-        <f>Main!J2</f>
-        <v>0</v>
-      </c>
-      <c r="K2" s="1">
-        <f>Main!K2</f>
-        <v>0</v>
-      </c>
-      <c r="L2" s="1">
-        <f>Main!L2</f>
-        <v>0</v>
-      </c>
-      <c r="M2" s="1">
-        <f>Main!M2</f>
-        <v>0</v>
-      </c>
-      <c r="N2" s="1">
-        <f>Main!N2</f>
-        <v>0</v>
-      </c>
-      <c r="O2" s="1">
-        <f>Main!O2</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="n">
+        <f aca="false">Main!B2</f>
+        <v>0</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <f aca="false">Main!C2</f>
+        <v>0</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <f aca="false">Main!D2</f>
+        <v>0</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <f aca="false">Main!E2</f>
+        <v>0</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <f aca="false">Main!F2</f>
+        <v>0</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <f aca="false">Main!G2</f>
+        <v>0</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <f aca="false">Main!H2</f>
+        <v>0</v>
+      </c>
+      <c r="I2" s="1" t="n">
+        <f aca="false">Main!I2</f>
+        <v>0</v>
+      </c>
+      <c r="J2" s="1" t="n">
+        <f aca="false">Main!J2</f>
+        <v>0</v>
+      </c>
+      <c r="K2" s="1" t="n">
+        <f aca="false">Main!K2</f>
+        <v>0</v>
+      </c>
+      <c r="L2" s="1" t="n">
+        <f aca="false">Main!L2</f>
+        <v>0</v>
+      </c>
+      <c r="M2" s="1" t="n">
+        <f aca="false">Main!M2</f>
+        <v>0</v>
+      </c>
+      <c r="N2" s="1" t="n">
+        <f aca="false">Main!N2</f>
+        <v>0</v>
+      </c>
+      <c r="O2" s="1" t="n">
+        <f aca="false">Main!O2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>37</v>
       </c>
@@ -1461,7 +1522,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D13" s="1" t="s">
         <v>44</v>
       </c>
@@ -1477,35 +1538,43 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A11" r:id="rId1"/>
+    <hyperlink ref="A11" r:id="rId1" display="http://cybuild.devpress.net"/>
   </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:O48"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="30.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="20.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="48.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="41.42578125" style="1" customWidth="1"/>
-    <col min="6" max="7" width="47.28515625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="43.28515625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="30.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="48.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="43" style="1" customWidth="1"/>
-    <col min="12" max="12" width="41.7109375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="47.28515625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="35.5703125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="10.5703125" style="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="48.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="47.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="43.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="48.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="41.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="47.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="35.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="10.57"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -1552,79 +1621,84 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="5"/>
     </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N24" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N26" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="34" spans="12:15" x14ac:dyDescent="0.25">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N34" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="37" spans="12:15" x14ac:dyDescent="0.25">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N37" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="12:15" x14ac:dyDescent="0.25">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N43" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="46" spans="12:15" x14ac:dyDescent="0.25">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N46" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="48" spans="12:15" x14ac:dyDescent="0.25">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L48" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M48" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="N48" s="1" t="s">
         <v>57</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="L48" r:id="rId1"/>
-    <hyperlink ref="M48" r:id="rId2"/>
+    <hyperlink ref="L48" r:id="rId1" display="engineer.27may2025@yopmail.com/Test@123"/>
+    <hyperlink ref="M48" r:id="rId2" display="technicaladmin.27may2025@yopmail.com/Test@123"/>
   </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Latest cahnges on 10Sept2026
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -1,19 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="5"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="3"/>
   </bookViews>
   <sheets>
-    <sheet name="configMobile" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="permitFlow" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="testFlow" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Main" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="configMobile" sheetId="1" r:id="rId1"/>
+    <sheet name="permitFlow" sheetId="2" r:id="rId2"/>
+    <sheet name="testFlow" sheetId="3" r:id="rId3"/>
+    <sheet name="Main" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="144525" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,198 +24,194 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="61">
   <si>
-    <t xml:space="preserve">Device Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Platform Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Platform Version</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Automation Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skip Unlock</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVD Launch Timeout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ensure Webview Have Pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Native Web Screenshot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New Command Timeout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Connect Hardware Keyboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unicoded Keyboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reset Keyboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No Reset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App Package</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App Activity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adb Exec Timeout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Client Company</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sdk_gphone64_x86_64</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Android</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UiAutomator2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">true</t>
-  </si>
-  <si>
-    <t xml:space="preserve">false</t>
-  </si>
-  <si>
-    <t xml:space="preserve">com.app.acompletions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">com.commissioning.ui.splash.SplashActivity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Android SDK built for x86</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pixel C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redmi26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.1.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Environment URL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L2 User Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permit Holder Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L4 User Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PCO User Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permit Approver (L4) Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Projectr Admin Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Discipline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://cybuild.devpress.net</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brave</t>
-  </si>
-  <si>
-    <t xml:space="preserve">todd.beck@example.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">julie.cole@example.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">noah.poulsen@example.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Julie Cole</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dhaval.barot@indianic.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tom@mac-24.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">john@mac-24.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kevin@mac-24.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Niall Stenson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QA Manager Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project Admin Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supervisor Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Engineer Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Technical Admin Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Admin Credentials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://im-aam.com/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://staging.im-aam.com/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">acompletions@admin.com/123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">admin@cybuild.com.au/Commsite12#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">engineer.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">technicaladmin.27may2025@yopmail.com/Test@123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E&amp;IC</t>
+    <t>Device Name</t>
+  </si>
+  <si>
+    <t>Platform Name</t>
+  </si>
+  <si>
+    <t>Platform Version</t>
+  </si>
+  <si>
+    <t>Automation Name</t>
+  </si>
+  <si>
+    <t>Skip Unlock</t>
+  </si>
+  <si>
+    <t>AVD Launch Timeout</t>
+  </si>
+  <si>
+    <t>Ensure Webview Have Pages</t>
+  </si>
+  <si>
+    <t>Native Web Screenshot</t>
+  </si>
+  <si>
+    <t>New Command Timeout</t>
+  </si>
+  <si>
+    <t>Connect Hardware Keyboard</t>
+  </si>
+  <si>
+    <t>Unicoded Keyboard</t>
+  </si>
+  <si>
+    <t>Reset Keyboard</t>
+  </si>
+  <si>
+    <t>No Reset</t>
+  </si>
+  <si>
+    <t>App Package</t>
+  </si>
+  <si>
+    <t>App Activity</t>
+  </si>
+  <si>
+    <t>Adb Exec Timeout</t>
+  </si>
+  <si>
+    <t>Client Company</t>
+  </si>
+  <si>
+    <t>sdk_gphone64_x86_64</t>
+  </si>
+  <si>
+    <t>Android</t>
+  </si>
+  <si>
+    <t>UiAutomator2</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t>com.app.acompletions</t>
+  </si>
+  <si>
+    <t>com.commissioning.ui.splash.SplashActivity</t>
+  </si>
+  <si>
+    <t>Android SDK built for x86</t>
+  </si>
+  <si>
+    <t>Pixel C</t>
+  </si>
+  <si>
+    <t>Redmi26</t>
+  </si>
+  <si>
+    <t>8.1.0</t>
+  </si>
+  <si>
+    <t>Environment URL</t>
+  </si>
+  <si>
+    <t>Project Name</t>
+  </si>
+  <si>
+    <t>L2 User Credentials</t>
+  </si>
+  <si>
+    <t>Permit Holder Credentials</t>
+  </si>
+  <si>
+    <t>L4 User Credentials</t>
+  </si>
+  <si>
+    <t>PCO User Credentials</t>
+  </si>
+  <si>
+    <t>Permit Approver (L4) Name</t>
+  </si>
+  <si>
+    <t>Projectr Admin Credentials</t>
+  </si>
+  <si>
+    <t>Discipline</t>
+  </si>
+  <si>
+    <t>http://cybuild.devpress.net</t>
+  </si>
+  <si>
+    <t>Brave</t>
+  </si>
+  <si>
+    <t>todd.beck@example.com/123456</t>
+  </si>
+  <si>
+    <t>julie.cole@example.com/123456</t>
+  </si>
+  <si>
+    <t>noah.poulsen@example.com/123456</t>
+  </si>
+  <si>
+    <t>Julie Cole</t>
+  </si>
+  <si>
+    <t>dhaval.barot@indianic.com/123456</t>
+  </si>
+  <si>
+    <t>tom@mac-24.com/Test@123</t>
+  </si>
+  <si>
+    <t>john@mac-24.com/123456</t>
+  </si>
+  <si>
+    <t>kevin@mac-24.com/123456</t>
+  </si>
+  <si>
+    <t>Niall Stenson</t>
+  </si>
+  <si>
+    <t>QA Manager Credentials</t>
+  </si>
+  <si>
+    <t>Project Admin Credentials</t>
+  </si>
+  <si>
+    <t>Supervisor Credentials</t>
+  </si>
+  <si>
+    <t>Engineer Credentials</t>
+  </si>
+  <si>
+    <t>Technical Admin Credentials</t>
+  </si>
+  <si>
+    <t>Super Admin Credentials</t>
+  </si>
+  <si>
+    <t>https://im-aam.com/</t>
+  </si>
+  <si>
+    <t>https://staging.im-aam.com/</t>
+  </si>
+  <si>
+    <t>acompletions@admin.com/123456</t>
+  </si>
+  <si>
+    <t>admin@cybuild.com.au/Commsite12#</t>
+  </si>
+  <si>
+    <t>engineer.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>technicaladmin.27may2025@yopmail.com/Test@123</t>
+  </si>
+  <si>
+    <t>E&amp;IC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="@"/>
-  </numFmts>
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -225,22 +220,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -248,7 +228,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <u val="single"/>
+      <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
@@ -265,84 +245,47 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -401,13 +344,26 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -449,12 +405,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -486,7 +442,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -510,7 +466,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -570,42 +526,41 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q35"/>
-  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="22.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="26.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="18.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="21.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="15.14"/>
+    <col min="1" max="1" width="23.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="27" style="1" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="22.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="26.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15" style="1" customWidth="1"/>
+    <col min="13" max="13" width="9" style="1" customWidth="1"/>
+    <col min="14" max="14" width="21.5703125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="41" style="1" customWidth="1"/>
+    <col min="16" max="16" width="17" style="1" customWidth="1"/>
+    <col min="17" max="17" width="15.140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -658,14 +613,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="1">
         <v>14</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -674,7 +629,7 @@
       <c r="E2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="1">
         <v>300000</v>
       </c>
       <c r="G2" s="4" t="s">
@@ -683,7 +638,7 @@
       <c r="H2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="1" t="n">
+      <c r="I2" s="1">
         <v>3600</v>
       </c>
       <c r="J2" s="4" t="s">
@@ -704,27 +659,27 @@
       <c r="O2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="P2" s="1" t="n">
+      <c r="P2" s="1">
         <v>60000</v>
       </c>
-      <c r="Q2" s="1" t="n">
-        <f aca="false">Main!B2</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C3" s="1" t="n">
+      <c r="Q2" s="1">
+        <f>Main!B2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C3" s="1">
         <v>12</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="1">
         <v>13</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -733,7 +688,7 @@
       <c r="E4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="1">
         <v>300000</v>
       </c>
       <c r="G4" s="4" t="s">
@@ -742,7 +697,7 @@
       <c r="H4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="1" t="n">
+      <c r="I4" s="1">
         <v>3600</v>
       </c>
       <c r="J4" s="4" t="s">
@@ -764,19 +719,19 @@
         <v>23</v>
       </c>
       <c r="P4" s="4"/>
-      <c r="Q4" s="1" t="n">
-        <f aca="false">Main!B4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Q4" s="1">
+        <f>Main!B4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C6" s="1">
         <v>11</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -785,7 +740,7 @@
       <c r="E6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="F6" s="1">
         <v>300000</v>
       </c>
       <c r="G6" s="4" t="s">
@@ -794,7 +749,7 @@
       <c r="H6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="1" t="n">
+      <c r="I6" s="1">
         <v>3600</v>
       </c>
       <c r="J6" s="4" t="s">
@@ -817,14 +772,14 @@
       </c>
       <c r="P6" s="4"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="C10" s="1">
         <v>13</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -833,7 +788,7 @@
       <c r="E10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="1" t="n">
+      <c r="F10" s="1">
         <v>300000</v>
       </c>
       <c r="G10" s="4" t="s">
@@ -842,7 +797,7 @@
       <c r="H10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I10" s="1" t="n">
+      <c r="I10" s="1">
         <v>3600</v>
       </c>
       <c r="J10" s="4" t="s">
@@ -865,14 +820,14 @@
       </c>
       <c r="P10" s="4"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="1" t="n">
+      <c r="C14" s="1">
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -881,7 +836,7 @@
       <c r="E14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F14" s="1" t="n">
+      <c r="F14" s="1">
         <v>300000</v>
       </c>
       <c r="G14" s="4" t="s">
@@ -890,7 +845,7 @@
       <c r="H14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="1" t="n">
+      <c r="I14" s="1">
         <v>3600</v>
       </c>
       <c r="J14" s="4" t="s">
@@ -913,14 +868,14 @@
       </c>
       <c r="P14" s="4"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="1" t="n">
+      <c r="C20" s="1">
         <v>13</v>
       </c>
       <c r="D20" s="1" t="s">
@@ -929,7 +884,7 @@
       <c r="E20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F20" s="1" t="n">
+      <c r="F20" s="1">
         <v>300000</v>
       </c>
       <c r="G20" s="4" t="s">
@@ -938,7 +893,7 @@
       <c r="H20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I20" s="1" t="n">
+      <c r="I20" s="1">
         <v>3600</v>
       </c>
       <c r="J20" s="4" t="s">
@@ -961,14 +916,14 @@
       </c>
       <c r="P20" s="4"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C23" s="1" t="n">
+      <c r="C23" s="1">
         <v>13</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -977,7 +932,7 @@
       <c r="E23" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F23" s="1" t="n">
+      <c r="F23" s="1">
         <v>300000</v>
       </c>
       <c r="G23" s="4" t="s">
@@ -986,7 +941,7 @@
       <c r="H23" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I23" s="1" t="n">
+      <c r="I23" s="1">
         <v>3600</v>
       </c>
       <c r="J23" s="4" t="s">
@@ -1008,19 +963,19 @@
         <v>23</v>
       </c>
       <c r="P23" s="4"/>
-      <c r="Q23" s="1" t="n">
-        <f aca="false">Main!B23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Q23" s="1">
+        <f>Main!B23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="1" t="n">
+      <c r="C25" s="1">
         <v>12</v>
       </c>
       <c r="D25" s="1" t="s">
@@ -1029,7 +984,7 @@
       <c r="E25" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F25" s="1" t="n">
+      <c r="F25" s="1">
         <v>300000</v>
       </c>
       <c r="G25" s="4" t="s">
@@ -1038,7 +993,7 @@
       <c r="H25" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I25" s="1" t="n">
+      <c r="I25" s="1">
         <v>3600</v>
       </c>
       <c r="J25" s="4" t="s">
@@ -1061,7 +1016,7 @@
       </c>
       <c r="P25" s="4"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -1077,7 +1032,7 @@
       <c r="E28" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F28" s="1" t="n">
+      <c r="F28" s="1">
         <v>300000</v>
       </c>
       <c r="G28" s="4" t="s">
@@ -1086,7 +1041,7 @@
       <c r="H28" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I28" s="1" t="n">
+      <c r="I28" s="1">
         <v>3600</v>
       </c>
       <c r="J28" s="4" t="s">
@@ -1108,19 +1063,19 @@
         <v>23</v>
       </c>
       <c r="P28" s="4"/>
-      <c r="Q28" s="1" t="n">
-        <f aca="false">Main!B28</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Q28" s="1">
+        <f>Main!B28</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="1" t="n">
+      <c r="C33" s="1">
         <v>8</v>
       </c>
       <c r="D33" s="1" t="s">
@@ -1129,7 +1084,7 @@
       <c r="E33" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F33" s="1" t="n">
+      <c r="F33" s="1">
         <v>300000</v>
       </c>
       <c r="G33" s="4" t="s">
@@ -1138,7 +1093,7 @@
       <c r="H33" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I33" s="1" t="n">
+      <c r="I33" s="1">
         <v>3600</v>
       </c>
       <c r="J33" s="4" t="s">
@@ -1160,19 +1115,19 @@
         <v>23</v>
       </c>
       <c r="P33" s="4"/>
-      <c r="Q33" s="1" t="n">
-        <f aca="false">Main!B33</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Q33" s="1">
+        <f>Main!B33</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C35" s="1" t="n">
+      <c r="C35" s="1">
         <v>12</v>
       </c>
       <c r="D35" s="1" t="s">
@@ -1181,7 +1136,7 @@
       <c r="E35" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F35" s="1" t="n">
+      <c r="F35" s="1">
         <v>300000</v>
       </c>
       <c r="G35" s="4" t="s">
@@ -1190,7 +1145,7 @@
       <c r="H35" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I35" s="1" t="n">
+      <c r="I35" s="1">
         <v>3600</v>
       </c>
       <c r="J35" s="4" t="s">
@@ -1212,42 +1167,34 @@
         <v>23</v>
       </c>
       <c r="P35" s="4"/>
-      <c r="Q35" s="1" t="n">
-        <f aca="false">Main!B35</f>
+      <c r="Q35" s="1">
+        <f>Main!B35</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="31.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="30.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="34.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="30.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="46.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.71"/>
+    <col min="1" max="1" width="26.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="34.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="31.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="30.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="34.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="30.42578125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="46.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -1276,45 +1223,45 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
-        <f aca="false">Main!A2</f>
+        <f>Main!A2</f>
         <v>https://im-aam.com/</v>
       </c>
-      <c r="B2" s="1" t="n">
-        <f aca="false">Main!B2</f>
-        <v>0</v>
-      </c>
-      <c r="C2" s="1" t="n">
-        <f aca="false">Main!D2</f>
-        <v>0</v>
-      </c>
-      <c r="D2" s="1" t="n">
-        <f aca="false">Main!E2</f>
-        <v>0</v>
-      </c>
-      <c r="E2" s="1" t="n">
-        <f aca="false">Main!F2</f>
-        <v>0</v>
-      </c>
-      <c r="F2" s="1" t="n">
-        <f aca="false">Main!H2</f>
-        <v>0</v>
-      </c>
-      <c r="G2" s="1" t="n">
-        <f aca="false">Main!I2</f>
-        <v>0</v>
-      </c>
-      <c r="H2" s="1" t="n">
-        <f aca="false">Main!J2</f>
-        <v>0</v>
-      </c>
-      <c r="I2" s="1" t="n">
-        <f aca="false">Main!O2</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1">
+        <f>Main!B2</f>
+        <v>0</v>
+      </c>
+      <c r="C2" s="1">
+        <f>Main!D2</f>
+        <v>0</v>
+      </c>
+      <c r="D2" s="1">
+        <f>Main!E2</f>
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <f>Main!F2</f>
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <f>Main!H2</f>
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
+        <f>Main!I2</f>
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <f>Main!J2</f>
+        <v>0</v>
+      </c>
+      <c r="I2" s="1">
+        <f>Main!O2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>37</v>
       </c>
@@ -1337,7 +1284,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C13" s="1" t="s">
         <v>44</v>
       </c>
@@ -1353,43 +1300,35 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A11" r:id="rId1" display="http://cybuild.devpress.net"/>
+    <hyperlink ref="A11" r:id="rId1"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O13"/>
-  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="44.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="32.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="47.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="48.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="43.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="25.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="40.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="42.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="41.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="46.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="35.57"/>
+    <col min="1" max="1" width="30.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16" style="1" customWidth="1"/>
+    <col min="4" max="4" width="44.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="32.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="47.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="48.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="43.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="25.7109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="40.140625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="42.85546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="41.28515625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="46.7109375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="35.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -1436,69 +1375,69 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
-        <f aca="false">Main!A2</f>
+        <f>Main!A2</f>
         <v>https://im-aam.com/</v>
       </c>
-      <c r="B2" s="1" t="n">
-        <f aca="false">Main!B2</f>
-        <v>0</v>
-      </c>
-      <c r="C2" s="1" t="n">
-        <f aca="false">Main!C2</f>
-        <v>0</v>
-      </c>
-      <c r="D2" s="1" t="n">
-        <f aca="false">Main!D2</f>
-        <v>0</v>
-      </c>
-      <c r="E2" s="1" t="n">
-        <f aca="false">Main!E2</f>
-        <v>0</v>
-      </c>
-      <c r="F2" s="1" t="n">
-        <f aca="false">Main!F2</f>
-        <v>0</v>
-      </c>
-      <c r="G2" s="1" t="n">
-        <f aca="false">Main!G2</f>
-        <v>0</v>
-      </c>
-      <c r="H2" s="1" t="n">
-        <f aca="false">Main!H2</f>
-        <v>0</v>
-      </c>
-      <c r="I2" s="1" t="n">
-        <f aca="false">Main!I2</f>
-        <v>0</v>
-      </c>
-      <c r="J2" s="1" t="n">
-        <f aca="false">Main!J2</f>
-        <v>0</v>
-      </c>
-      <c r="K2" s="1" t="n">
-        <f aca="false">Main!K2</f>
-        <v>0</v>
-      </c>
-      <c r="L2" s="1" t="n">
-        <f aca="false">Main!L2</f>
-        <v>0</v>
-      </c>
-      <c r="M2" s="1" t="n">
-        <f aca="false">Main!M2</f>
-        <v>0</v>
-      </c>
-      <c r="N2" s="1" t="n">
-        <f aca="false">Main!N2</f>
-        <v>0</v>
-      </c>
-      <c r="O2" s="1" t="n">
-        <f aca="false">Main!O2</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1">
+        <f>Main!B2</f>
+        <v>0</v>
+      </c>
+      <c r="C2" s="1">
+        <f>Main!C2</f>
+        <v>0</v>
+      </c>
+      <c r="D2" s="1">
+        <f>Main!D2</f>
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <f>Main!E2</f>
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <f>Main!F2</f>
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
+        <f>Main!G2</f>
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <f>Main!H2</f>
+        <v>0</v>
+      </c>
+      <c r="I2" s="1">
+        <f>Main!I2</f>
+        <v>0</v>
+      </c>
+      <c r="J2" s="1">
+        <f>Main!J2</f>
+        <v>0</v>
+      </c>
+      <c r="K2" s="1">
+        <f>Main!K2</f>
+        <v>0</v>
+      </c>
+      <c r="L2" s="1">
+        <f>Main!L2</f>
+        <v>0</v>
+      </c>
+      <c r="M2" s="1">
+        <f>Main!M2</f>
+        <v>0</v>
+      </c>
+      <c r="N2" s="1">
+        <f>Main!N2</f>
+        <v>0</v>
+      </c>
+      <c r="O2" s="1">
+        <f>Main!O2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>37</v>
       </c>
@@ -1522,7 +1461,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D13" s="1" t="s">
         <v>44</v>
       </c>
@@ -1538,43 +1477,35 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A11" r:id="rId1" display="http://cybuild.devpress.net"/>
+    <hyperlink ref="A11" r:id="rId1"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O48"/>
-  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="48.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="47.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="43.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="48.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="41.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="47.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="35.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="10.57"/>
+    <col min="1" max="1" width="30.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="48.42578125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="41.42578125" style="1" customWidth="1"/>
+    <col min="6" max="7" width="47.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="43.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="30.42578125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="48.140625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="43" style="1" customWidth="1"/>
+    <col min="12" max="12" width="41.7109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="47.28515625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="35.5703125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="10.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -1621,60 +1552,60 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B19" s="5"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N24" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
       <c r="N26" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" spans="12:15" x14ac:dyDescent="0.25">
       <c r="N34" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" spans="12:15" x14ac:dyDescent="0.25">
       <c r="N37" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" spans="12:15" x14ac:dyDescent="0.25">
       <c r="N43" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" spans="12:15" x14ac:dyDescent="0.25">
       <c r="N46" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" spans="12:15" x14ac:dyDescent="0.25">
       <c r="L48" s="1" t="s">
         <v>58</v>
       </c>
@@ -1690,15 +1621,10 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="L48" r:id="rId1" display="engineer.27may2025@yopmail.com/Test@123"/>
-    <hyperlink ref="M48" r:id="rId2" display="technicaladmin.27may2025@yopmail.com/Test@123"/>
+    <hyperlink ref="L48" r:id="rId1"/>
+    <hyperlink ref="M48" r:id="rId2"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>